<commit_message>
data(proposal): 해외 상장 주식 다년 일봉 수집 (2026-09-20 05:07)
</commit_message>
<xml_diff>
--- a/고객제안서_자산배분.xlsx
+++ b/고객제안서_자산배분.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제안서" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="배분규칙" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자산군" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상품" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기대수익률" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="제안서" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="배분규칙" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="자산군" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="상품" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="출처" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="기대수익률" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="사용법" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'상품'!$A$7:$M$156</definedName>
@@ -1376,7 +1376,7 @@
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>유니버스 2026-09-20 01:05:58 · 문서 2026-09-20 01:08 (KST)</t>
+          <t>유니버스 2026-09-20 14:07:54 · 문서 2026-09-20 14:07 (KST)</t>
         </is>
       </c>
     </row>
@@ -2411,13 +2411,13 @@
         <v>99</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>0.1049382716049381</v>
+        <v>0.09780242562454644</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.2923973274425171</v>
+        <v>0.2921539773352639</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>-0.3235610824922673</v>
+        <v>-0.3237114148035969</v>
       </c>
     </row>
     <row r="12">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="F34" s="34" t="inlineStr">
         <is>
-          <t>932조원</t>
+          <t>931조원</t>
         </is>
       </c>
       <c r="G34" s="35" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="F39" s="28" t="inlineStr">
         <is>
-          <t>902조원</t>
+          <t>901조원</t>
         </is>
       </c>
       <c r="G39" s="30" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
-          <t>570조원</t>
+          <t>569조원</t>
         </is>
       </c>
       <c r="G40" s="35" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="F43" s="28" t="inlineStr">
         <is>
-          <t>1,177조원</t>
+          <t>1,176조원</t>
         </is>
       </c>
       <c r="G43" s="30" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="F45" s="28" t="inlineStr">
         <is>
-          <t>1,425조원</t>
+          <t>1,424조원</t>
         </is>
       </c>
       <c r="G45" s="30" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="C46" s="33" t="inlineStr">
         <is>
-          <t>골드만삭스</t>
+          <t>버크셔 해서웨이 B</t>
         </is>
       </c>
       <c r="D46" s="33" t="inlineStr">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
-          <t>380조원</t>
+          <t>1,511조원</t>
         </is>
       </c>
       <c r="G46" s="35" t="inlineStr">
@@ -5035,13 +5035,13 @@
         </is>
       </c>
       <c r="I46" s="36" t="n">
-        <v>0.2129</v>
+        <v>0.1287</v>
       </c>
       <c r="J46" s="36" t="n">
-        <v>0.2868</v>
+        <v>0.1716</v>
       </c>
       <c r="K46" s="37" t="n">
-        <v>-0.3284</v>
+        <v>-0.2658</v>
       </c>
       <c r="L46" s="34" t="inlineStr">
         <is>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="M46" s="38" t="inlineStr">
         <is>
-          <t>5해 연21.3% · 변동성 28.7% (위험대비 0.64) · 최대낙폭 -33% · 가장 나쁜 창 연20.9%</t>
+          <t>5해 연12.9% · 변동성 17.2% (위험대비 0.59) · 최대낙폭 -27% · 가장 나쁜 창 연3.5%</t>
         </is>
       </c>
     </row>
@@ -5067,12 +5067,12 @@
       </c>
       <c r="C47" s="14" t="inlineStr">
         <is>
-          <t>팔로알토네트웍스</t>
+          <t>골드만삭스</t>
         </is>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E47" s="14" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="F47" s="28" t="inlineStr">
         <is>
-          <t>412조원</t>
+          <t>380조원</t>
         </is>
       </c>
       <c r="G47" s="30" t="inlineStr">
@@ -5092,17 +5092,17 @@
       </c>
       <c r="H47" s="30" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I47" s="29" t="n">
-        <v>0.4321</v>
+        <v>0.2129</v>
       </c>
       <c r="J47" s="29" t="n">
-        <v>0.4356</v>
+        <v>0.2868</v>
       </c>
       <c r="K47" s="31" t="n">
-        <v>-0.3601</v>
+        <v>-0.3284</v>
       </c>
       <c r="L47" s="28" t="inlineStr">
         <is>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="M47" s="32" t="inlineStr">
         <is>
-          <t>3해 연43.2% · 변동성 43.6% (위험대비 0.93) · 최대낙폭 -36% · 가장 나쁜 창 연43.2%</t>
+          <t>5해 연21.3% · 변동성 28.7% (위험대비 0.64) · 최대낙폭 -33% · 가장 나쁜 창 연20.9%</t>
         </is>
       </c>
     </row>
@@ -5128,12 +5128,12 @@
       </c>
       <c r="C48" s="33" t="inlineStr">
         <is>
-          <t>버텍스</t>
+          <t>팔로알토네트웍스</t>
         </is>
       </c>
       <c r="D48" s="33" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E48" s="33" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="F48" s="34" t="inlineStr">
         <is>
-          <t>179조원</t>
+          <t>412조원</t>
         </is>
       </c>
       <c r="G48" s="35" t="inlineStr">
@@ -5153,17 +5153,17 @@
       </c>
       <c r="H48" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I48" s="36" t="n">
-        <v>0.2184</v>
+        <v>0.4321</v>
       </c>
       <c r="J48" s="36" t="n">
-        <v>0.2925</v>
+        <v>0.4356</v>
       </c>
       <c r="K48" s="37" t="n">
-        <v>-0.2907</v>
+        <v>-0.3601</v>
       </c>
       <c r="L48" s="34" t="inlineStr">
         <is>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="M48" s="38" t="inlineStr">
         <is>
-          <t>5해 연21.8% · 변동성 29.2% (위험대비 0.65) · 최대낙폭 -29% · 가장 나쁜 창 연13.5%</t>
+          <t>3해 연43.2% · 변동성 43.6% (위험대비 0.93) · 최대낙폭 -36% · 가장 나쁜 창 연43.2%</t>
         </is>
       </c>
     </row>
@@ -5189,12 +5189,12 @@
       </c>
       <c r="C49" s="14" t="inlineStr">
         <is>
-          <t>JP모간체이스</t>
+          <t>버텍스</t>
         </is>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -5204,7 +5204,7 @@
       </c>
       <c r="F49" s="28" t="inlineStr">
         <is>
-          <t>1,288조원</t>
+          <t>178조원</t>
         </is>
       </c>
       <c r="G49" s="30" t="inlineStr">
@@ -5218,13 +5218,13 @@
         </is>
       </c>
       <c r="I49" s="29" t="n">
-        <v>0.2019</v>
+        <v>0.2184</v>
       </c>
       <c r="J49" s="29" t="n">
-        <v>0.2436</v>
+        <v>0.2925</v>
       </c>
       <c r="K49" s="31" t="n">
-        <v>-0.3877</v>
+        <v>-0.2907</v>
       </c>
       <c r="L49" s="28" t="inlineStr">
         <is>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="M49" s="32" t="inlineStr">
         <is>
-          <t>5해 연20.2% · 변동성 24.4% (위험대비 0.71) · 최대낙폭 -39% · 가장 나쁜 창 연14.3%</t>
+          <t>5해 연21.8% · 변동성 29.2% (위험대비 0.65) · 최대낙폭 -29% · 가장 나쁜 창 연13.5%</t>
         </is>
       </c>
     </row>
@@ -5250,12 +5250,12 @@
       </c>
       <c r="C50" s="33" t="inlineStr">
         <is>
-          <t>애플</t>
+          <t>JP모간체이스</t>
         </is>
       </c>
       <c r="D50" s="33" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E50" s="33" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
-          <t>6,799조원</t>
+          <t>1,287조원</t>
         </is>
       </c>
       <c r="G50" s="35" t="inlineStr">
@@ -5279,13 +5279,13 @@
         </is>
       </c>
       <c r="I50" s="36" t="n">
-        <v>0.1818</v>
+        <v>0.2019</v>
       </c>
       <c r="J50" s="36" t="n">
-        <v>0.2794</v>
+        <v>0.2436</v>
       </c>
       <c r="K50" s="37" t="n">
-        <v>-0.3336</v>
+        <v>-0.3877</v>
       </c>
       <c r="L50" s="34" t="inlineStr">
         <is>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="M50" s="38" t="inlineStr">
         <is>
-          <t>5해 연18.2% · 변동성 27.9% (위험대비 0.55) · 최대낙폭 -33% · 가장 나쁜 창 연18.2%</t>
+          <t>5해 연20.2% · 변동성 24.4% (위험대비 0.71) · 최대낙폭 -39% · 가장 나쁜 창 연14.3%</t>
         </is>
       </c>
     </row>
@@ -5311,12 +5311,12 @@
       </c>
       <c r="C51" s="14" t="inlineStr">
         <is>
-          <t>비자</t>
+          <t>애플</t>
         </is>
       </c>
       <c r="D51" s="14" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="F51" s="28" t="inlineStr">
         <is>
-          <t>958조원</t>
+          <t>6,794조원</t>
         </is>
       </c>
       <c r="G51" s="30" t="inlineStr">
@@ -5340,13 +5340,13 @@
         </is>
       </c>
       <c r="I51" s="29" t="n">
-        <v>0.1116</v>
+        <v>0.1818</v>
       </c>
       <c r="J51" s="29" t="n">
-        <v>0.2287</v>
+        <v>0.2794</v>
       </c>
       <c r="K51" s="31" t="n">
-        <v>-0.2414</v>
+        <v>-0.3336</v>
       </c>
       <c r="L51" s="28" t="inlineStr">
         <is>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="M51" s="32" t="inlineStr">
         <is>
-          <t>5해 연11.2% · 변동성 22.9% (위험대비 0.37) · 최대낙폭 -24% · 가장 나쁜 창 연7.2%</t>
+          <t>5해 연18.2% · 변동성 27.9% (위험대비 0.55) · 최대낙폭 -33% · 가장 나쁜 창 연18.2%</t>
         </is>
       </c>
     </row>
@@ -5372,12 +5372,12 @@
       </c>
       <c r="C52" s="33" t="inlineStr">
         <is>
-          <t>이튼</t>
+          <t>비자</t>
         </is>
       </c>
       <c r="D52" s="33" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E52" s="33" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
-          <t>229조원</t>
+          <t>958조원</t>
         </is>
       </c>
       <c r="G52" s="35" t="inlineStr">
@@ -5401,13 +5401,13 @@
         </is>
       </c>
       <c r="I52" s="36" t="n">
-        <v>0.2329</v>
+        <v>0.1116</v>
       </c>
       <c r="J52" s="36" t="n">
-        <v>0.3206</v>
+        <v>0.2287</v>
       </c>
       <c r="K52" s="37" t="n">
-        <v>-0.3446</v>
+        <v>-0.2414</v>
       </c>
       <c r="L52" s="34" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="M52" s="38" t="inlineStr">
         <is>
-          <t>5해 연23.3% · 변동성 32.1% (위험대비 0.64) · 최대낙폭 -34% · 가장 나쁜 창 연18.2%</t>
+          <t>5해 연11.2% · 변동성 22.9% (위험대비 0.37) · 최대낙폭 -24% · 가장 나쁜 창 연7.2%</t>
         </is>
       </c>
     </row>
@@ -5433,12 +5433,12 @@
       </c>
       <c r="C53" s="14" t="inlineStr">
         <is>
-          <t>모간스탠리</t>
+          <t>이튼</t>
         </is>
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>산업재</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="F53" s="28" t="inlineStr">
         <is>
-          <t>441조원</t>
+          <t>228조원</t>
         </is>
       </c>
       <c r="G53" s="30" t="inlineStr">
@@ -5462,13 +5462,13 @@
         </is>
       </c>
       <c r="I53" s="29" t="n">
-        <v>0.1797</v>
+        <v>0.2329</v>
       </c>
       <c r="J53" s="29" t="n">
-        <v>0.2889</v>
+        <v>0.3206</v>
       </c>
       <c r="K53" s="31" t="n">
-        <v>-0.3238</v>
+        <v>-0.3446</v>
       </c>
       <c r="L53" s="28" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="M53" s="32" t="inlineStr">
         <is>
-          <t>5해 연18.0% · 변동성 28.9% (위험대비 0.52) · 최대낙폭 -32% · 가장 나쁜 창 연18.0%</t>
+          <t>5해 연23.3% · 변동성 32.1% (위험대비 0.64) · 최대낙폭 -34% · 가장 나쁜 창 연18.2%</t>
         </is>
       </c>
     </row>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="C54" s="33" t="inlineStr">
         <is>
-          <t>프로그레시브</t>
+          <t>모간스탠리</t>
         </is>
       </c>
       <c r="D54" s="33" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
-          <t>172조원</t>
+          <t>441조원</t>
         </is>
       </c>
       <c r="G54" s="35" t="inlineStr">
@@ -5523,13 +5523,13 @@
         </is>
       </c>
       <c r="I54" s="36" t="n">
-        <v>0.2061</v>
+        <v>0.1797</v>
       </c>
       <c r="J54" s="36" t="n">
-        <v>0.2553</v>
+        <v>0.2889</v>
       </c>
       <c r="K54" s="37" t="n">
-        <v>-0.3035</v>
+        <v>-0.3238</v>
       </c>
       <c r="L54" s="34" t="inlineStr">
         <is>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="M54" s="38" t="inlineStr">
         <is>
-          <t>5해 연20.6% · 변동성 25.5% (위험대비 0.70) · 최대낙폭 -30% · 가장 나쁜 창 연-6.7%</t>
+          <t>5해 연18.0% · 변동성 28.9% (위험대비 0.52) · 최대낙폭 -32% · 가장 나쁜 창 연18.0%</t>
         </is>
       </c>
     </row>
@@ -5555,12 +5555,12 @@
       </c>
       <c r="C55" s="14" t="inlineStr">
         <is>
-          <t>록히드마틴</t>
+          <t>프로그레시브</t>
         </is>
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="F55" s="28" t="inlineStr">
         <is>
-          <t>171조원</t>
+          <t>172조원</t>
         </is>
       </c>
       <c r="G55" s="30" t="inlineStr">
@@ -5584,13 +5584,13 @@
         </is>
       </c>
       <c r="I55" s="29" t="n">
-        <v>0.1195</v>
+        <v>0.2061</v>
       </c>
       <c r="J55" s="29" t="n">
-        <v>0.2409</v>
+        <v>0.2553</v>
       </c>
       <c r="K55" s="31" t="n">
-        <v>-0.3179</v>
+        <v>-0.3035</v>
       </c>
       <c r="L55" s="28" t="inlineStr">
         <is>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M55" s="32" t="inlineStr">
         <is>
-          <t>5해 연11.9% · 변동성 24.1% (위험대비 0.38) · 최대낙폭 -32% · 가장 나쁜 창 연11.1%</t>
+          <t>5해 연20.6% · 변동성 25.5% (위험대비 0.70) · 최대낙폭 -30% · 가장 나쁜 창 연-6.7%</t>
         </is>
       </c>
     </row>
@@ -5616,12 +5616,12 @@
       </c>
       <c r="C56" s="33" t="inlineStr">
         <is>
-          <t>시스코</t>
+          <t>록히드마틴</t>
         </is>
       </c>
       <c r="D56" s="33" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>산업재</t>
         </is>
       </c>
       <c r="E56" s="33" t="inlineStr">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
-          <t>598조원</t>
+          <t>170조원</t>
         </is>
       </c>
       <c r="G56" s="35" t="inlineStr">
@@ -5645,13 +5645,13 @@
         </is>
       </c>
       <c r="I56" s="36" t="n">
-        <v>0.1674</v>
+        <v>0.1195</v>
       </c>
       <c r="J56" s="36" t="n">
-        <v>0.2597</v>
+        <v>0.2409</v>
       </c>
       <c r="K56" s="37" t="n">
-        <v>-0.3668</v>
+        <v>-0.3179</v>
       </c>
       <c r="L56" s="34" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="M56" s="38" t="inlineStr">
         <is>
-          <t>5해 연16.7% · 변동성 26.0% (위험대비 0.54) · 최대낙폭 -37% · 가장 나쁜 창 연16.7%</t>
+          <t>5해 연11.9% · 변동성 24.1% (위험대비 0.38) · 최대낙폭 -32% · 가장 나쁜 창 연11.1%</t>
         </is>
       </c>
     </row>
@@ -12128,7 +12128,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E7" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
data(proposal): 원/달러 일별 환율 수집 (2026-09-20 05:35)
</commit_message>
<xml_diff>
--- a/고객제안서_자산배분.xlsx
+++ b/고객제안서_자산배분.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제안서" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="배분규칙" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자산군" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상품" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기대수익률" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="제안서" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="배분규칙" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="자산군" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="상품" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="출처" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="기대수익률" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="사용법" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'상품'!$A$6:$M$156</definedName>
@@ -1043,7 +1043,7 @@
         <v/>
       </c>
       <c r="G22" s="17" t="n">
-        <v>0.0621</v>
+        <v>0.0561</v>
       </c>
       <c r="H22" s="15">
         <f>IF(ISNUMBER($F22),$F22,0)</f>
@@ -1376,7 +1376,7 @@
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>유니버스 2026-09-20 14:07:54 · 문서 2026-09-20 14:10 (KST)</t>
+          <t>유니버스 2026-09-20 14:35:38 · 문서 2026-09-20 14:35 (KST)</t>
         </is>
       </c>
     </row>
@@ -4181,13 +4181,13 @@
         </is>
       </c>
       <c r="I32" s="36" t="n">
-        <v>0.2423</v>
+        <v>0.2862</v>
       </c>
       <c r="J32" s="36" t="n">
-        <v>0.2345</v>
+        <v>0.2527</v>
       </c>
       <c r="K32" s="37" t="n">
-        <v>-0.2192</v>
+        <v>-0.2288</v>
       </c>
       <c r="L32" s="34" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="M32" s="38" t="inlineStr">
         <is>
-          <t>5해 연24.2% · 변동성 23.4% (위험대비 0.91) · 최대낙폭 -22% · 가장 나쁜 창 연23.2%</t>
+          <t>5해 연28.6% · 변동성 25.3% (위험대비 1.02) · 최대낙폭 -23% · 가장 나쁜 창 연24.1%</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t>필립모리스</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="D33" s="14" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="F33" s="28" t="inlineStr">
         <is>
-          <t>407조원</t>
+          <t>526조원</t>
         </is>
       </c>
       <c r="G33" s="30" t="inlineStr">
@@ -4242,13 +4242,13 @@
         </is>
       </c>
       <c r="I33" s="29" t="n">
-        <v>0.1805</v>
+        <v>0.1704</v>
       </c>
       <c r="J33" s="29" t="n">
-        <v>0.233</v>
+        <v>0.1891</v>
       </c>
       <c r="K33" s="31" t="n">
-        <v>-0.2278</v>
+        <v>-0.1672</v>
       </c>
       <c r="L33" s="28" t="inlineStr">
         <is>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="M33" s="32" t="inlineStr">
         <is>
-          <t>5해 연18.1% · 변동성 23.3% (위험대비 0.65) · 최대낙폭 -23% · 가장 나쁜 창 연17.5%</t>
+          <t>5해 연17.0% · 변동성 18.9% (위험대비 0.75) · 최대낙폭 -17% · 가장 나쁜 창 연17.0%</t>
         </is>
       </c>
     </row>
@@ -4274,12 +4274,12 @@
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
-          <t>엑슨모빌</t>
+          <t>길리어드</t>
         </is>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
-          <t>에너지</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="E34" s="33" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="F34" s="34" t="inlineStr">
         <is>
-          <t>931조원</t>
+          <t>258조원</t>
         </is>
       </c>
       <c r="G34" s="35" t="inlineStr">
@@ -4303,13 +4303,13 @@
         </is>
       </c>
       <c r="I34" s="36" t="n">
-        <v>0.2897</v>
+        <v>0.2477</v>
       </c>
       <c r="J34" s="36" t="n">
-        <v>0.2671</v>
+        <v>0.263</v>
       </c>
       <c r="K34" s="37" t="n">
-        <v>-0.2051</v>
+        <v>-0.2465</v>
       </c>
       <c r="L34" s="34" t="inlineStr">
         <is>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="M34" s="38" t="inlineStr">
         <is>
-          <t>5해 연29.0% · 변동성 26.7% (위험대비 0.98) · 최대낙폭 -21% · 가장 나쁜 창 연15.4%</t>
+          <t>5해 연24.8% · 변동성 26.3% (위험대비 0.83) · 최대낙폭 -25% · 가장 나쁜 창 연24.8%</t>
         </is>
       </c>
     </row>
@@ -4335,12 +4335,12 @@
       </c>
       <c r="C35" s="14" t="inlineStr">
         <is>
-          <t>길리어드</t>
+          <t>필립모리스</t>
         </is>
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>필수소비재</t>
         </is>
       </c>
       <c r="E35" s="14" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="F35" s="28" t="inlineStr">
         <is>
-          <t>258조원</t>
+          <t>407조원</t>
         </is>
       </c>
       <c r="G35" s="30" t="inlineStr">
@@ -4364,13 +4364,13 @@
         </is>
       </c>
       <c r="I35" s="29" t="n">
-        <v>0.2051</v>
+        <v>0.2222</v>
       </c>
       <c r="J35" s="29" t="n">
-        <v>0.2461</v>
+        <v>0.2438</v>
       </c>
       <c r="K35" s="31" t="n">
-        <v>-0.2659</v>
+        <v>-0.184</v>
       </c>
       <c r="L35" s="28" t="inlineStr">
         <is>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="M35" s="32" t="inlineStr">
         <is>
-          <t>5해 연20.5% · 변동성 24.6% (위험대비 0.72) · 최대낙폭 -27% · 가장 나쁜 창 연20.5%</t>
+          <t>5해 연22.2% · 변동성 24.4% (위험대비 0.80) · 최대낙폭 -18% · 가장 나쁜 창 연18.3%</t>
         </is>
       </c>
     </row>
@@ -4396,12 +4396,12 @@
       </c>
       <c r="C36" s="33" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>엑슨모빌</t>
         </is>
       </c>
       <c r="D36" s="33" t="inlineStr">
         <is>
-          <t>필수소비재</t>
+          <t>에너지</t>
         </is>
       </c>
       <c r="E36" s="33" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="F36" s="34" t="inlineStr">
         <is>
-          <t>526조원</t>
+          <t>931조원</t>
         </is>
       </c>
       <c r="G36" s="35" t="inlineStr">
@@ -4425,13 +4425,13 @@
         </is>
       </c>
       <c r="I36" s="36" t="n">
-        <v>0.1304</v>
+        <v>0.3352000000000001</v>
       </c>
       <c r="J36" s="36" t="n">
-        <v>0.1665</v>
+        <v>0.2815</v>
       </c>
       <c r="K36" s="37" t="n">
-        <v>-0.1727</v>
+        <v>-0.2045</v>
       </c>
       <c r="L36" s="34" t="inlineStr">
         <is>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="M36" s="38" t="inlineStr">
         <is>
-          <t>5해 연13.0% · 변동성 16.6% (위험대비 0.61) · 최대낙폭 -17% · 가장 나쁜 창 연13.0%</t>
+          <t>5해 연33.5% · 변동성 28.1% (위험대비 1.09) · 최대낙폭 -20% · 가장 나쁜 창 연17.1%</t>
         </is>
       </c>
     </row>
@@ -4457,12 +4457,12 @@
       </c>
       <c r="C37" s="14" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>처브</t>
         </is>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E37" s="14" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="F37" s="28" t="inlineStr">
         <is>
-          <t>362조원</t>
+          <t>182조원</t>
         </is>
       </c>
       <c r="G37" s="30" t="inlineStr">
@@ -4486,13 +4486,13 @@
         </is>
       </c>
       <c r="I37" s="29" t="n">
-        <v>0.2098</v>
+        <v>0.1934</v>
       </c>
       <c r="J37" s="29" t="n">
-        <v>0.2431</v>
+        <v>0.2271</v>
       </c>
       <c r="K37" s="31" t="n">
-        <v>-0.3284</v>
+        <v>-0.2158</v>
       </c>
       <c r="L37" s="28" t="inlineStr">
         <is>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="M37" s="32" t="inlineStr">
         <is>
-          <t>5해 연21.0% · 변동성 24.3% (위험대비 0.75) · 최대낙폭 -33% · 가장 나쁜 창 연21.0%</t>
+          <t>5해 연19.3% · 변동성 22.7% (위험대비 0.73) · 최대낙폭 -22% · 가장 나쁜 창 연19.3%</t>
         </is>
       </c>
     </row>
@@ -4518,12 +4518,12 @@
       </c>
       <c r="C38" s="33" t="inlineStr">
         <is>
-          <t>처브</t>
+          <t>존슨앤드존슨</t>
         </is>
       </c>
       <c r="D38" s="33" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="E38" s="33" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
-          <t>182조원</t>
+          <t>901조원</t>
         </is>
       </c>
       <c r="G38" s="35" t="inlineStr">
@@ -4547,13 +4547,13 @@
         </is>
       </c>
       <c r="I38" s="36" t="n">
-        <v>0.1527</v>
+        <v>0.1715</v>
       </c>
       <c r="J38" s="36" t="n">
-        <v>0.2041</v>
+        <v>0.2006</v>
       </c>
       <c r="K38" s="37" t="n">
-        <v>-0.1926</v>
+        <v>-0.2108</v>
       </c>
       <c r="L38" s="34" t="inlineStr">
         <is>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="M38" s="38" t="inlineStr">
         <is>
-          <t>5해 연15.3% · 변동성 20.4% (위험대비 0.61) · 최대낙폭 -19% · 가장 나쁜 창 연15.3%</t>
+          <t>5해 연17.1% · 변동성 20.1% (위험대비 0.71) · 최대낙폭 -21% · 가장 나쁜 창 연17.1%</t>
         </is>
       </c>
     </row>
@@ -4579,12 +4579,12 @@
       </c>
       <c r="C39" s="14" t="inlineStr">
         <is>
-          <t>존슨앤드존슨</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>산업재</t>
         </is>
       </c>
       <c r="E39" s="14" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="F39" s="28" t="inlineStr">
         <is>
-          <t>901조원</t>
+          <t>362조원</t>
         </is>
       </c>
       <c r="G39" s="30" t="inlineStr">
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="I39" s="29" t="n">
-        <v>0.1315</v>
+        <v>0.2526</v>
       </c>
       <c r="J39" s="29" t="n">
-        <v>0.1756</v>
+        <v>0.2634</v>
       </c>
       <c r="K39" s="31" t="n">
-        <v>-0.1841</v>
+        <v>-0.317</v>
       </c>
       <c r="L39" s="28" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="M39" s="32" t="inlineStr">
         <is>
-          <t>5해 연13.2% · 변동성 17.6% (위험대비 0.59) · 최대낙폭 -18% · 가장 나쁜 창 연13.2%</t>
+          <t>5해 연25.3% · 변동성 26.3% (위험대비 0.85) · 최대낙폭 -32% · 가장 나쁜 창 연25.2%</t>
         </is>
       </c>
     </row>
@@ -4640,12 +4640,12 @@
       </c>
       <c r="C40" s="33" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>JP모간체이스</t>
         </is>
       </c>
       <c r="D40" s="33" t="inlineStr">
         <is>
-          <t>에너지</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E40" s="33" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
-          <t>569조원</t>
+          <t>1,287조원</t>
         </is>
       </c>
       <c r="G40" s="35" t="inlineStr">
@@ -4669,13 +4669,13 @@
         </is>
       </c>
       <c r="I40" s="36" t="n">
-        <v>0.2156</v>
+        <v>0.2444</v>
       </c>
       <c r="J40" s="36" t="n">
-        <v>0.2528</v>
+        <v>0.254</v>
       </c>
       <c r="K40" s="37" t="n">
-        <v>-0.2495</v>
+        <v>-0.2822</v>
       </c>
       <c r="L40" s="34" t="inlineStr">
         <is>
@@ -4684,7 +4684,7 @@
       </c>
       <c r="M40" s="38" t="inlineStr">
         <is>
-          <t>5해 연21.6% · 변동성 25.3% (위험대비 0.74) · 최대낙폭 -25% · 가장 나쁜 창 연12.6%</t>
+          <t>5해 연24.4% · 변동성 25.4% (위험대비 0.85) · 최대낙폭 -28% · 가장 나쁜 창 연15.1%</t>
         </is>
       </c>
     </row>
@@ -4701,12 +4701,12 @@
       </c>
       <c r="C41" s="14" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>필수소비재</t>
+          <t>에너지</t>
         </is>
       </c>
       <c r="E41" s="14" t="inlineStr">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="F41" s="28" t="inlineStr">
         <is>
-          <t>161조원</t>
+          <t>569조원</t>
         </is>
       </c>
       <c r="G41" s="30" t="inlineStr">
@@ -4730,13 +4730,13 @@
         </is>
       </c>
       <c r="I41" s="29" t="n">
-        <v>0.1542</v>
+        <v>0.2585</v>
       </c>
       <c r="J41" s="29" t="n">
-        <v>0.2167</v>
+        <v>0.2673</v>
       </c>
       <c r="K41" s="31" t="n">
-        <v>-0.2583</v>
+        <v>-0.2604</v>
       </c>
       <c r="L41" s="28" t="inlineStr">
         <is>
@@ -4745,7 +4745,7 @@
       </c>
       <c r="M41" s="32" t="inlineStr">
         <is>
-          <t>5해 연15.4% · 변동성 21.7% (위험대비 0.58) · 최대낙폭 -26% · 가장 나쁜 창 연13.3%</t>
+          <t>5해 연25.9% · 변동성 26.7% (위험대비 0.86) · 최대낙폭 -26% · 가장 나쁜 창 연14.2%</t>
         </is>
       </c>
     </row>
@@ -4762,12 +4762,12 @@
       </c>
       <c r="C42" s="33" t="inlineStr">
         <is>
-          <t>캐터필러</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="D42" s="33" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>필수소비재</t>
         </is>
       </c>
       <c r="E42" s="33" t="inlineStr">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
-          <t>515조원</t>
+          <t>161조원</t>
         </is>
       </c>
       <c r="G42" s="35" t="inlineStr">
@@ -4791,13 +4791,13 @@
         </is>
       </c>
       <c r="I42" s="36" t="n">
-        <v>0.3371</v>
+        <v>0.195</v>
       </c>
       <c r="J42" s="36" t="n">
-        <v>0.3169</v>
+        <v>0.2341</v>
       </c>
       <c r="K42" s="37" t="n">
-        <v>-0.3405</v>
+        <v>-0.2366</v>
       </c>
       <c r="L42" s="34" t="inlineStr">
         <is>
@@ -4806,7 +4806,7 @@
       </c>
       <c r="M42" s="38" t="inlineStr">
         <is>
-          <t>5해 연33.7% · 변동성 31.7% (위험대비 0.98) · 최대낙폭 -34% · 가장 나쁜 창 연33.7%</t>
+          <t>5해 연19.5% · 변동성 23.4% (위험대비 0.71) · 최대낙폭 -24% · 가장 나쁜 창 연14.1%</t>
         </is>
       </c>
     </row>
@@ -4823,12 +4823,12 @@
       </c>
       <c r="C43" s="14" t="inlineStr">
         <is>
-          <t>월마트</t>
+          <t>버크셔 해서웨이 B</t>
         </is>
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>필수소비재</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E43" s="14" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="F43" s="28" t="inlineStr">
         <is>
-          <t>1,176조원</t>
+          <t>1,511조원</t>
         </is>
       </c>
       <c r="G43" s="30" t="inlineStr">
@@ -4852,13 +4852,13 @@
         </is>
       </c>
       <c r="I43" s="29" t="n">
-        <v>0.1836</v>
+        <v>0.1686</v>
       </c>
       <c r="J43" s="29" t="n">
-        <v>0.2249</v>
+        <v>0.1924</v>
       </c>
       <c r="K43" s="31" t="n">
-        <v>-0.2574</v>
+        <v>-0.2123</v>
       </c>
       <c r="L43" s="28" t="inlineStr">
         <is>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="M43" s="32" t="inlineStr">
         <is>
-          <t>5해 연18.4% · 변동성 22.5% (위험대비 0.69) · 최대낙폭 -26% · 가장 나쁜 창 연3.0%</t>
+          <t>5해 연16.9% · 변동성 19.2% (위험대비 0.73) · 최대낙폭 -21% · 가장 나쁜 창 연4.2%</t>
         </is>
       </c>
     </row>
@@ -4884,12 +4884,12 @@
       </c>
       <c r="C44" s="33" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>골드만삭스</t>
         </is>
       </c>
       <c r="D44" s="33" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E44" s="33" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="F44" s="34" t="inlineStr">
         <is>
-          <t>289조원</t>
+          <t>380조원</t>
         </is>
       </c>
       <c r="G44" s="35" t="inlineStr">
@@ -4913,13 +4913,13 @@
         </is>
       </c>
       <c r="I44" s="36" t="n">
-        <v>0.1601</v>
+        <v>0.2557</v>
       </c>
       <c r="J44" s="36" t="n">
-        <v>0.2458</v>
+        <v>0.2923</v>
       </c>
       <c r="K44" s="37" t="n">
-        <v>-0.2486</v>
+        <v>-0.2931</v>
       </c>
       <c r="L44" s="34" t="inlineStr">
         <is>
@@ -4928,7 +4928,7 @@
       </c>
       <c r="M44" s="38" t="inlineStr">
         <is>
-          <t>5해 연16.0% · 변동성 24.6% (위험대비 0.54) · 최대낙폭 -25% · 가장 나쁜 창 연16.0%</t>
+          <t>5해 연25.6% · 변동성 29.2% (위험대비 0.78) · 최대낙폭 -29% · 가장 나쁜 창 연21.7%</t>
         </is>
       </c>
     </row>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="C45" s="14" t="inlineStr">
         <is>
-          <t>일라이 릴리</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="D45" s="14" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="F45" s="28" t="inlineStr">
         <is>
-          <t>1,424조원</t>
+          <t>289조원</t>
         </is>
       </c>
       <c r="G45" s="30" t="inlineStr">
@@ -4974,13 +4974,13 @@
         </is>
       </c>
       <c r="I45" s="29" t="n">
-        <v>0.3799</v>
+        <v>0.2011</v>
       </c>
       <c r="J45" s="29" t="n">
-        <v>0.3256</v>
+        <v>0.2618</v>
       </c>
       <c r="K45" s="31" t="n">
-        <v>-0.3448</v>
+        <v>-0.2882</v>
       </c>
       <c r="L45" s="28" t="inlineStr">
         <is>
@@ -4989,7 +4989,7 @@
       </c>
       <c r="M45" s="32" t="inlineStr">
         <is>
-          <t>5해 연38.0% · 변동성 32.6% (위험대비 1.08) · 최대낙폭 -34% · 가장 나쁜 창 연25.1%</t>
+          <t>5해 연20.1% · 변동성 26.2% (위험대비 0.66) · 최대낙폭 -29% · 가장 나쁜 창 연19.6%</t>
         </is>
       </c>
     </row>
@@ -5006,12 +5006,12 @@
       </c>
       <c r="C46" s="33" t="inlineStr">
         <is>
-          <t>버크셔 해서웨이 B</t>
+          <t>캐터필러</t>
         </is>
       </c>
       <c r="D46" s="33" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>산업재</t>
         </is>
       </c>
       <c r="E46" s="33" t="inlineStr">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
-          <t>1,511조원</t>
+          <t>515조원</t>
         </is>
       </c>
       <c r="G46" s="35" t="inlineStr">
@@ -5035,13 +5035,13 @@
         </is>
       </c>
       <c r="I46" s="36" t="n">
-        <v>0.1287</v>
+        <v>0.3844</v>
       </c>
       <c r="J46" s="36" t="n">
-        <v>0.1716</v>
+        <v>0.3214</v>
       </c>
       <c r="K46" s="37" t="n">
-        <v>-0.2658</v>
+        <v>-0.3597</v>
       </c>
       <c r="L46" s="34" t="inlineStr">
         <is>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="M46" s="38" t="inlineStr">
         <is>
-          <t>5해 연12.9% · 변동성 17.2% (위험대비 0.59) · 최대낙폭 -27% · 가장 나쁜 창 연3.5%</t>
+          <t>5해 연38.4% · 변동성 32.1% (위험대비 1.11) · 최대낙폭 -36% · 가장 나쁜 창 연38.4%</t>
         </is>
       </c>
     </row>
@@ -5067,12 +5067,12 @@
       </c>
       <c r="C47" s="14" t="inlineStr">
         <is>
-          <t>골드만삭스</t>
+          <t>일라이 릴리</t>
         </is>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="E47" s="14" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="F47" s="28" t="inlineStr">
         <is>
-          <t>380조원</t>
+          <t>1,424조원</t>
         </is>
       </c>
       <c r="G47" s="30" t="inlineStr">
@@ -5096,13 +5096,13 @@
         </is>
       </c>
       <c r="I47" s="29" t="n">
-        <v>0.2129</v>
+        <v>0.4287</v>
       </c>
       <c r="J47" s="29" t="n">
-        <v>0.2868</v>
+        <v>0.3434</v>
       </c>
       <c r="K47" s="31" t="n">
-        <v>-0.3284</v>
+        <v>-0.357</v>
       </c>
       <c r="L47" s="28" t="inlineStr">
         <is>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="M47" s="32" t="inlineStr">
         <is>
-          <t>5해 연21.3% · 변동성 28.7% (위험대비 0.64) · 최대낙폭 -33% · 가장 나쁜 창 연20.9%</t>
+          <t>5해 연42.9% · 변동성 34.3% (위험대비 1.17) · 최대낙폭 -36% · 가장 나쁜 창 연26.9%</t>
         </is>
       </c>
     </row>
@@ -5128,12 +5128,12 @@
       </c>
       <c r="C48" s="33" t="inlineStr">
         <is>
-          <t>팔로알토네트웍스</t>
+          <t>월마트</t>
         </is>
       </c>
       <c r="D48" s="33" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>필수소비재</t>
         </is>
       </c>
       <c r="E48" s="33" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="F48" s="34" t="inlineStr">
         <is>
-          <t>412조원</t>
+          <t>1,176조원</t>
         </is>
       </c>
       <c r="G48" s="35" t="inlineStr">
@@ -5153,17 +5153,17 @@
       </c>
       <c r="H48" s="35" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I48" s="36" t="n">
-        <v>0.4321</v>
+        <v>0.2255</v>
       </c>
       <c r="J48" s="36" t="n">
-        <v>0.4356</v>
+        <v>0.245</v>
       </c>
       <c r="K48" s="37" t="n">
-        <v>-0.3601</v>
+        <v>-0.2999</v>
       </c>
       <c r="L48" s="34" t="inlineStr">
         <is>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="M48" s="38" t="inlineStr">
         <is>
-          <t>3해 연43.2% · 변동성 43.6% (위험대비 0.93) · 최대낙폭 -36% · 가장 나쁜 창 연43.2%</t>
+          <t>5해 연22.6% · 변동성 24.5% (위험대비 0.81) · 최대낙폭 -30% · 가장 나쁜 창 연3.7%</t>
         </is>
       </c>
     </row>
@@ -5189,12 +5189,12 @@
       </c>
       <c r="C49" s="14" t="inlineStr">
         <is>
-          <t>버텍스</t>
+          <t>시스코</t>
         </is>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -5204,7 +5204,7 @@
       </c>
       <c r="F49" s="28" t="inlineStr">
         <is>
-          <t>178조원</t>
+          <t>598조원</t>
         </is>
       </c>
       <c r="G49" s="30" t="inlineStr">
@@ -5218,13 +5218,13 @@
         </is>
       </c>
       <c r="I49" s="29" t="n">
-        <v>0.2184</v>
+        <v>0.2087</v>
       </c>
       <c r="J49" s="29" t="n">
-        <v>0.2925</v>
+        <v>0.2738</v>
       </c>
       <c r="K49" s="31" t="n">
-        <v>-0.2907</v>
+        <v>-0.2894</v>
       </c>
       <c r="L49" s="28" t="inlineStr">
         <is>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="M49" s="32" t="inlineStr">
         <is>
-          <t>5해 연21.8% · 변동성 29.2% (위험대비 0.65) · 최대낙폭 -29% · 가장 나쁜 창 연13.5%</t>
+          <t>5해 연20.9% · 변동성 27.4% (위험대비 0.66) · 최대낙폭 -29% · 가장 나쁜 창 연20.9%</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5250,7 @@
       </c>
       <c r="C50" s="33" t="inlineStr">
         <is>
-          <t>JP모간체이스</t>
+          <t>비자</t>
         </is>
       </c>
       <c r="D50" s="33" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
-          <t>1,287조원</t>
+          <t>958조원</t>
         </is>
       </c>
       <c r="G50" s="35" t="inlineStr">
@@ -5279,13 +5279,13 @@
         </is>
       </c>
       <c r="I50" s="36" t="n">
-        <v>0.2019</v>
+        <v>0.1509</v>
       </c>
       <c r="J50" s="36" t="n">
-        <v>0.2436</v>
+        <v>0.2408</v>
       </c>
       <c r="K50" s="37" t="n">
-        <v>-0.3877</v>
+        <v>-0.1856</v>
       </c>
       <c r="L50" s="34" t="inlineStr">
         <is>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="M50" s="38" t="inlineStr">
         <is>
-          <t>5해 연20.2% · 변동성 24.4% (위험대비 0.71) · 최대낙폭 -39% · 가장 나쁜 창 연14.3%</t>
+          <t>5해 연15.1% · 변동성 24.1% (위험대비 0.51) · 최대낙폭 -19% · 가장 나쁜 창 연8.0%</t>
         </is>
       </c>
     </row>
@@ -5311,12 +5311,12 @@
       </c>
       <c r="C51" s="14" t="inlineStr">
         <is>
-          <t>애플</t>
+          <t>모간스탠리</t>
         </is>
       </c>
       <c r="D51" s="14" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="F51" s="28" t="inlineStr">
         <is>
-          <t>6,794조원</t>
+          <t>441조원</t>
         </is>
       </c>
       <c r="G51" s="30" t="inlineStr">
@@ -5340,13 +5340,13 @@
         </is>
       </c>
       <c r="I51" s="29" t="n">
-        <v>0.1818</v>
+        <v>0.2214</v>
       </c>
       <c r="J51" s="29" t="n">
-        <v>0.2794</v>
+        <v>0.2919</v>
       </c>
       <c r="K51" s="31" t="n">
-        <v>-0.3336</v>
+        <v>-0.2937</v>
       </c>
       <c r="L51" s="28" t="inlineStr">
         <is>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="M51" s="32" t="inlineStr">
         <is>
-          <t>5해 연18.2% · 변동성 27.9% (위험대비 0.55) · 최대낙폭 -33% · 가장 나쁜 창 연18.2%</t>
+          <t>5해 연22.1% · 변동성 29.2% (위험대비 0.66) · 최대낙폭 -29% · 가장 나쁜 창 연22.1%</t>
         </is>
       </c>
     </row>
@@ -5372,12 +5372,12 @@
       </c>
       <c r="C52" s="33" t="inlineStr">
         <is>
-          <t>비자</t>
+          <t>팔로알토네트웍스</t>
         </is>
       </c>
       <c r="D52" s="33" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E52" s="33" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
-          <t>958조원</t>
+          <t>412조원</t>
         </is>
       </c>
       <c r="G52" s="35" t="inlineStr">
@@ -5397,17 +5397,17 @@
       </c>
       <c r="H52" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I52" s="36" t="n">
-        <v>0.1116</v>
+        <v>0.453</v>
       </c>
       <c r="J52" s="36" t="n">
-        <v>0.2287</v>
+        <v>0.4484</v>
       </c>
       <c r="K52" s="37" t="n">
-        <v>-0.2414</v>
+        <v>-0.3606</v>
       </c>
       <c r="L52" s="34" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="M52" s="38" t="inlineStr">
         <is>
-          <t>5해 연11.2% · 변동성 22.9% (위험대비 0.37) · 최대낙폭 -24% · 가장 나쁜 창 연7.2%</t>
+          <t>3해 연45.3% · 변동성 44.8% (위험대비 0.95) · 최대낙폭 -36% · 가장 나쁜 창 연45.3%</t>
         </is>
       </c>
     </row>
@@ -5433,12 +5433,12 @@
       </c>
       <c r="C53" s="14" t="inlineStr">
         <is>
-          <t>이튼</t>
+          <t>애플</t>
         </is>
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="F53" s="28" t="inlineStr">
         <is>
-          <t>228조원</t>
+          <t>6,794조원</t>
         </is>
       </c>
       <c r="G53" s="30" t="inlineStr">
@@ -5462,13 +5462,13 @@
         </is>
       </c>
       <c r="I53" s="29" t="n">
-        <v>0.2329</v>
+        <v>0.2236</v>
       </c>
       <c r="J53" s="29" t="n">
-        <v>0.3206</v>
+        <v>0.291</v>
       </c>
       <c r="K53" s="31" t="n">
-        <v>-0.3446</v>
+        <v>-0.3245</v>
       </c>
       <c r="L53" s="28" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="M53" s="32" t="inlineStr">
         <is>
-          <t>5해 연23.3% · 변동성 32.1% (위험대비 0.64) · 최대낙폭 -34% · 가장 나쁜 창 연18.2%</t>
+          <t>5해 연22.4% · 변동성 29.1% (위험대비 0.67) · 최대낙폭 -32% · 가장 나쁜 창 연22.4%</t>
         </is>
       </c>
     </row>
@@ -5494,12 +5494,12 @@
       </c>
       <c r="C54" s="33" t="inlineStr">
         <is>
-          <t>모간스탠리</t>
+          <t>버텍스</t>
         </is>
       </c>
       <c r="D54" s="33" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="E54" s="33" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
-          <t>441조원</t>
+          <t>178조원</t>
         </is>
       </c>
       <c r="G54" s="35" t="inlineStr">
@@ -5523,13 +5523,13 @@
         </is>
       </c>
       <c r="I54" s="36" t="n">
-        <v>0.1797</v>
+        <v>0.2614</v>
       </c>
       <c r="J54" s="36" t="n">
-        <v>0.2889</v>
+        <v>0.3027</v>
       </c>
       <c r="K54" s="37" t="n">
-        <v>-0.3238</v>
+        <v>-0.3211</v>
       </c>
       <c r="L54" s="34" t="inlineStr">
         <is>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="M54" s="38" t="inlineStr">
         <is>
-          <t>5해 연18.0% · 변동성 28.9% (위험대비 0.52) · 최대낙폭 -32% · 가장 나쁜 창 연18.0%</t>
+          <t>5해 연26.1% · 변동성 30.3% (위험대비 0.77) · 최대낙폭 -32% · 가장 나쁜 창 연15.2%</t>
         </is>
       </c>
     </row>
@@ -5555,12 +5555,12 @@
       </c>
       <c r="C55" s="14" t="inlineStr">
         <is>
-          <t>프로그레시브</t>
+          <t>유니온퍼시픽</t>
         </is>
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>산업재</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="F55" s="28" t="inlineStr">
         <is>
-          <t>172조원</t>
+          <t>230조원</t>
         </is>
       </c>
       <c r="G55" s="30" t="inlineStr">
@@ -5584,13 +5584,13 @@
         </is>
       </c>
       <c r="I55" s="29" t="n">
-        <v>0.2061</v>
+        <v>0.1232</v>
       </c>
       <c r="J55" s="29" t="n">
-        <v>0.2553</v>
+        <v>0.2429</v>
       </c>
       <c r="K55" s="31" t="n">
-        <v>-0.3035</v>
+        <v>-0.2736</v>
       </c>
       <c r="L55" s="28" t="inlineStr">
         <is>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M55" s="32" t="inlineStr">
         <is>
-          <t>5해 연20.6% · 변동성 25.5% (위험대비 0.70) · 최대낙폭 -30% · 가장 나쁜 창 연-6.7%</t>
+          <t>5해 연12.3% · 변동성 24.3% (위험대비 0.39) · 최대낙폭 -27% · 가장 나쁜 창 연12.3%</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="C56" s="33" t="inlineStr">
         <is>
-          <t>록히드마틴</t>
+          <t>GE에어로스페이스</t>
         </is>
       </c>
       <c r="D56" s="33" t="inlineStr">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
-          <t>170조원</t>
+          <t>452조원</t>
         </is>
       </c>
       <c r="G56" s="35" t="inlineStr">
@@ -5645,13 +5645,13 @@
         </is>
       </c>
       <c r="I56" s="36" t="n">
-        <v>0.1195</v>
+        <v>0.4306</v>
       </c>
       <c r="J56" s="36" t="n">
-        <v>0.2409</v>
+        <v>0.3175</v>
       </c>
       <c r="K56" s="37" t="n">
-        <v>-0.3179</v>
+        <v>-0.383</v>
       </c>
       <c r="L56" s="34" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="M56" s="38" t="inlineStr">
         <is>
-          <t>5해 연11.9% · 변동성 24.1% (위험대비 0.38) · 최대낙폭 -32% · 가장 나쁜 창 연11.1%</t>
+          <t>5해 연43.1% · 변동성 31.8% (위험대비 1.27) · 최대낙폭 -38% · 가장 나쁜 창 연9.8%</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>SOL 미국S&amp;P500</t>
+          <t>ACE 미국나스닥100미국채혼합50액티브</t>
         </is>
       </c>
       <c r="D83" s="14" t="inlineStr">
@@ -7247,12 +7247,12 @@
       </c>
       <c r="E83" s="14" t="inlineStr">
         <is>
-          <t>신한자산운용</t>
+          <t>한국투자신탁운용</t>
         </is>
       </c>
       <c r="F83" s="28" t="inlineStr">
         <is>
-          <t>2,987억원</t>
+          <t>9,455억원</t>
         </is>
       </c>
       <c r="G83" s="30" t="inlineStr">
@@ -7266,20 +7266,20 @@
         </is>
       </c>
       <c r="I83" s="29" t="n">
-        <v>0.2146</v>
+        <v>0.1323</v>
       </c>
       <c r="J83" s="29" t="n">
-        <v>0.1556</v>
+        <v>0.09820000000000001</v>
       </c>
       <c r="K83" s="31" t="n">
-        <v>-0.1924</v>
+        <v>-0.1486</v>
       </c>
       <c r="L83" s="39" t="n">
-        <v>4.7e-05</v>
+        <v>0.0015</v>
       </c>
       <c r="M83" s="32" t="inlineStr">
         <is>
-          <t>3해 연21.5% · 변동성 15.6% (위험대비 1.20) · 최대낙폭 -19% · 보수 0.00% · 가장 나쁜 창 연16.8%</t>
+          <t>3해 연13.2% · 변동성 9.8% (위험대비 1.06) · 최대낙폭 -15% · 보수 0.15% · 가장 나쁜 창 연11.6%</t>
         </is>
       </c>
     </row>
@@ -7296,7 +7296,7 @@
       </c>
       <c r="C84" s="33" t="inlineStr">
         <is>
-          <t>ACE 미국배당다우존스</t>
+          <t>SOL 미국S&amp;P500</t>
         </is>
       </c>
       <c r="D84" s="33" t="inlineStr">
@@ -7306,12 +7306,12 @@
       </c>
       <c r="E84" s="33" t="inlineStr">
         <is>
-          <t>한국투신운용(ETF)</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
-          <t>9,703억원</t>
+          <t>2,987억원</t>
         </is>
       </c>
       <c r="G84" s="35" t="inlineStr">
@@ -7325,20 +7325,20 @@
         </is>
       </c>
       <c r="I84" s="36" t="n">
-        <v>0.1576</v>
+        <v>0.2146</v>
       </c>
       <c r="J84" s="36" t="n">
-        <v>0.1409</v>
+        <v>0.1556</v>
       </c>
       <c r="K84" s="37" t="n">
-        <v>-0.1321</v>
+        <v>-0.1924</v>
       </c>
       <c r="L84" s="40" t="n">
-        <v>0.0001</v>
+        <v>4.7e-05</v>
       </c>
       <c r="M84" s="38" t="inlineStr">
         <is>
-          <t>3해 연15.8% · 변동성 14.1% (위험대비 0.92) · 최대낙폭 -13% · 보수 0.01% · 가장 나쁜 창 연15.8%</t>
+          <t>3해 연21.5% · 변동성 15.6% (위험대비 1.20) · 최대낙폭 -19% · 보수 0.00% · 가장 나쁜 창 연16.8%</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="C85" s="14" t="inlineStr">
         <is>
-          <t>ACE 미국나스닥100미국채혼합50액티브</t>
+          <t>SOL 미국TOP5채권혼합50</t>
         </is>
       </c>
       <c r="D85" s="14" t="inlineStr">
@@ -7365,12 +7365,12 @@
       </c>
       <c r="E85" s="14" t="inlineStr">
         <is>
-          <t>한국투자신탁운용</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="F85" s="28" t="inlineStr">
         <is>
-          <t>9,455억원</t>
+          <t>1,248억원</t>
         </is>
       </c>
       <c r="G85" s="30" t="inlineStr">
@@ -7384,20 +7384,20 @@
         </is>
       </c>
       <c r="I85" s="29" t="n">
-        <v>0.1323</v>
+        <v>0.1197</v>
       </c>
       <c r="J85" s="29" t="n">
-        <v>0.09820000000000001</v>
+        <v>0.098</v>
       </c>
       <c r="K85" s="31" t="n">
-        <v>-0.1486</v>
+        <v>-0.113</v>
       </c>
       <c r="L85" s="39" t="n">
-        <v>0.0015</v>
+        <v>0.0025</v>
       </c>
       <c r="M85" s="32" t="inlineStr">
         <is>
-          <t>3해 연13.2% · 변동성 9.8% (위험대비 1.06) · 최대낙폭 -15% · 보수 0.15% · 가장 나쁜 창 연11.6%</t>
+          <t>3해 연12.0% · 변동성 9.8% (위험대비 0.93) · 최대낙폭 -11% · 보수 0.25% · 가장 나쁜 창 연11.9%</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C86" s="33" t="inlineStr">
         <is>
-          <t>SOL 미국TOP5채권혼합50</t>
+          <t>ACE 미국배당다우존스</t>
         </is>
       </c>
       <c r="D86" s="33" t="inlineStr">
@@ -7424,12 +7424,12 @@
       </c>
       <c r="E86" s="33" t="inlineStr">
         <is>
-          <t>신한자산운용</t>
+          <t>한국투신운용(ETF)</t>
         </is>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
-          <t>1,248억원</t>
+          <t>9,703억원</t>
         </is>
       </c>
       <c r="G86" s="35" t="inlineStr">
@@ -7443,20 +7443,20 @@
         </is>
       </c>
       <c r="I86" s="36" t="n">
-        <v>0.1197</v>
+        <v>0.1576</v>
       </c>
       <c r="J86" s="36" t="n">
-        <v>0.098</v>
+        <v>0.1409</v>
       </c>
       <c r="K86" s="37" t="n">
-        <v>-0.113</v>
+        <v>-0.1321</v>
       </c>
       <c r="L86" s="40" t="n">
-        <v>0.0025</v>
+        <v>0.0001</v>
       </c>
       <c r="M86" s="38" t="inlineStr">
         <is>
-          <t>3해 연12.0% · 변동성 9.8% (위험대비 0.93) · 최대낙폭 -11% · 보수 0.25% · 가장 나쁜 창 연11.9%</t>
+          <t>3해 연15.8% · 변동성 14.1% (위험대비 0.92) · 최대낙폭 -13% · 보수 0.01% · 가장 나쁜 창 연15.8%</t>
         </is>
       </c>
     </row>
@@ -7473,22 +7473,22 @@
       </c>
       <c r="C87" s="14" t="inlineStr">
         <is>
-          <t>KODEX 미국배당커버드콜액티브</t>
+          <t>ACE 엔비디아채권혼합</t>
         </is>
       </c>
       <c r="D87" s="14" t="inlineStr">
         <is>
-          <t>커버드콜</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="E87" s="14" t="inlineStr">
         <is>
-          <t>삼성자산운용(ETF)</t>
+          <t>한국투신운용(ETF)</t>
         </is>
       </c>
       <c r="F87" s="28" t="inlineStr">
         <is>
-          <t>2조원</t>
+          <t>2,464억원</t>
         </is>
       </c>
       <c r="G87" s="30" t="inlineStr">
@@ -7502,20 +7502,20 @@
         </is>
       </c>
       <c r="I87" s="29" t="n">
-        <v>0.1642</v>
+        <v>0.222</v>
       </c>
       <c r="J87" s="29" t="n">
-        <v>0.1268</v>
+        <v>0.1681</v>
       </c>
       <c r="K87" s="31" t="n">
-        <v>-0.137</v>
+        <v>-0.139</v>
       </c>
       <c r="L87" s="39" t="n">
-        <v>0.0019</v>
+        <v>0.0007000000000000001</v>
       </c>
       <c r="M87" s="32" t="inlineStr">
         <is>
-          <t>3해 연16.4% · 변동성 12.7% (위험대비 1.07) · 최대낙폭 -14% · 보수 0.19% · 가장 나쁜 창 연14.1%</t>
+          <t>3해 연22.2% · 변동성 16.8% (위험대비 1.15) · 최대낙폭 -14% · 보수 0.07% · 가장 나쁜 창 연9.9%</t>
         </is>
       </c>
     </row>
@@ -7532,22 +7532,22 @@
       </c>
       <c r="C88" s="33" t="inlineStr">
         <is>
-          <t>ACE 엔비디아채권혼합</t>
+          <t>KODEX 미국배당커버드콜액티브</t>
         </is>
       </c>
       <c r="D88" s="33" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>커버드콜</t>
         </is>
       </c>
       <c r="E88" s="33" t="inlineStr">
         <is>
-          <t>한국투신운용(ETF)</t>
+          <t>삼성자산운용(ETF)</t>
         </is>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
-          <t>2,464억원</t>
+          <t>2조원</t>
         </is>
       </c>
       <c r="G88" s="35" t="inlineStr">
@@ -7561,20 +7561,20 @@
         </is>
       </c>
       <c r="I88" s="36" t="n">
-        <v>0.222</v>
+        <v>0.1642</v>
       </c>
       <c r="J88" s="36" t="n">
-        <v>0.1681</v>
+        <v>0.1268</v>
       </c>
       <c r="K88" s="37" t="n">
-        <v>-0.139</v>
+        <v>-0.137</v>
       </c>
       <c r="L88" s="40" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.0019</v>
       </c>
       <c r="M88" s="38" t="inlineStr">
         <is>
-          <t>3해 연22.2% · 변동성 16.8% (위험대비 1.15) · 최대낙폭 -14% · 보수 0.07% · 가장 나쁜 창 연9.9%</t>
+          <t>3해 연16.4% · 변동성 12.7% (위험대비 1.07) · 최대낙폭 -14% · 보수 0.19% · 가장 나쁜 창 연14.1%</t>
         </is>
       </c>
     </row>
@@ -7650,7 +7650,7 @@
       </c>
       <c r="C90" s="33" t="inlineStr">
         <is>
-          <t>ACE 글로벌인컴TOP10</t>
+          <t>TIGER 일본니케이225</t>
         </is>
       </c>
       <c r="D90" s="33" t="inlineStr">
@@ -7660,12 +7660,12 @@
       </c>
       <c r="E90" s="33" t="inlineStr">
         <is>
-          <t>한국투신운용(ETF)</t>
+          <t>미래에셋자산운용</t>
         </is>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
-          <t>854억원</t>
+          <t>3,967억원</t>
         </is>
       </c>
       <c r="G90" s="35" t="inlineStr">
@@ -7675,24 +7675,24 @@
       </c>
       <c r="H90" s="35" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I90" s="36" t="n">
-        <v>0.0969</v>
+        <v>0.1541</v>
       </c>
       <c r="J90" s="36" t="n">
-        <v>0.09880000000000001</v>
+        <v>0.2107</v>
       </c>
       <c r="K90" s="37" t="n">
-        <v>-0.141</v>
+        <v>-0.2394</v>
       </c>
       <c r="L90" s="40" t="n">
-        <v>0.0024</v>
+        <v>0.0035</v>
       </c>
       <c r="M90" s="38" t="inlineStr">
         <is>
-          <t>3해 연9.7% · 변동성 9.9% (위험대비 0.70) · 최대낙폭 -14% · 보수 0.24% · 가장 나쁜 창 연6.0%</t>
+          <t>5해 연15.4% · 변동성 21.1% (위험대비 0.60) · 최대낙폭 -24% · 보수 0.35% · 가장 나쁜 창 연15.4%</t>
         </is>
       </c>
     </row>
@@ -7709,7 +7709,7 @@
       </c>
       <c r="C91" s="14" t="inlineStr">
         <is>
-          <t>KODEX MSCI선진국</t>
+          <t>TIGER 테슬라채권혼합Fn</t>
         </is>
       </c>
       <c r="D91" s="14" t="inlineStr">
@@ -7719,12 +7719,12 @@
       </c>
       <c r="E91" s="14" t="inlineStr">
         <is>
-          <t>삼성자산운용(ETF)</t>
+          <t>미래에셋자산운용</t>
         </is>
       </c>
       <c r="F91" s="28" t="inlineStr">
         <is>
-          <t>4,989억원</t>
+          <t>4,393억원</t>
         </is>
       </c>
       <c r="G91" s="30" t="inlineStr">
@@ -7734,24 +7734,24 @@
       </c>
       <c r="H91" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I91" s="29" t="n">
-        <v>0.1505</v>
+        <v>0.0867</v>
       </c>
       <c r="J91" s="29" t="n">
-        <v>0.1519</v>
+        <v>0.2019</v>
       </c>
       <c r="K91" s="31" t="n">
-        <v>-0.1646</v>
+        <v>-0.2107</v>
       </c>
       <c r="L91" s="39" t="n">
-        <v>0.003</v>
+        <v>0.0025</v>
       </c>
       <c r="M91" s="32" t="inlineStr">
         <is>
-          <t>5해 연15.1% · 변동성 15.2% (위험대비 0.81) · 최대낙폭 -16% · 보수 0.30% · 가장 나쁜 창 연15.1%</t>
+          <t>3해 연8.7% · 변동성 20.2% (위험대비 0.29) · 최대낙폭 -21% · 보수 0.25% · 가장 나쁜 창 연1.2%</t>
         </is>
       </c>
     </row>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="C92" s="33" t="inlineStr">
         <is>
-          <t>KODEX 미국나스닥AI테크액티브</t>
+          <t>ACE 미국30년국채액티브(H)</t>
         </is>
       </c>
       <c r="D92" s="33" t="inlineStr">
@@ -7778,12 +7778,12 @@
       </c>
       <c r="E92" s="33" t="inlineStr">
         <is>
-          <t>삼성자산운용(ETF)</t>
+          <t>한국투자신탁운용</t>
         </is>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
-          <t>1,282억원</t>
+          <t>1조원</t>
         </is>
       </c>
       <c r="G92" s="35" t="inlineStr">
@@ -7797,20 +7797,20 @@
         </is>
       </c>
       <c r="I92" s="36" t="n">
-        <v>0.4652000000000001</v>
+        <v>-0.0398</v>
       </c>
       <c r="J92" s="36" t="n">
-        <v>0.304</v>
+        <v>0.137</v>
       </c>
       <c r="K92" s="37" t="n">
-        <v>-0.3126</v>
+        <v>-0.1731</v>
       </c>
       <c r="L92" s="40" t="n">
-        <v>0.005</v>
+        <v>0.0005</v>
       </c>
       <c r="M92" s="38" t="inlineStr">
         <is>
-          <t>3해 연46.5% · 변동성 30.4% (위험대비 1.44) · 최대낙폭 -31% · 보수 0.50% · 가장 나쁜 창 연46.5%</t>
+          <t>3해 연-4.0% · 변동성 13.7% (위험대비 -0.50) · 최대낙폭 -17% · 보수 0.05% · 가장 나쁜 창 연-4.0%</t>
         </is>
       </c>
     </row>
@@ -7827,49 +7827,49 @@
       </c>
       <c r="C93" s="14" t="inlineStr">
         <is>
-          <t>ACE 미국달러SOFR금리(합성)</t>
+          <t>RISE 미국테크100데일리고정커버드콜</t>
         </is>
       </c>
       <c r="D93" s="14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>커버드콜</t>
         </is>
       </c>
       <c r="E93" s="14" t="inlineStr">
         <is>
-          <t>한국투신운용(ETF)</t>
+          <t>KB자산운용</t>
         </is>
       </c>
       <c r="F93" s="28" t="inlineStr">
         <is>
-          <t>3,365억원</t>
+          <t>5,772억원</t>
         </is>
       </c>
       <c r="G93" s="30" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H93" s="30" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I93" s="29" t="n">
-        <v>0.0626</v>
+        <v>0.2319</v>
       </c>
       <c r="J93" s="29" t="n">
-        <v>0.08869999999999999</v>
+        <v>0.1842</v>
       </c>
       <c r="K93" s="31" t="n">
-        <v>-0.1358</v>
+        <v>-0.1436</v>
       </c>
       <c r="L93" s="39" t="n">
-        <v>0.0005</v>
+        <v>0.0025</v>
       </c>
       <c r="M93" s="32" t="inlineStr">
         <is>
-          <t>3해 연6.3% · 변동성 8.9% (위험대비 0.39) · 최대낙폭 -14% · 보수 0.05% · 가장 나쁜 창 연3.1%</t>
+          <t>1해 연23.2% · 변동성 18.4% (위험대비 1.11) · 최대낙폭 -14% · 보수 0.25%</t>
         </is>
       </c>
     </row>
@@ -7886,7 +7886,7 @@
       </c>
       <c r="C94" s="33" t="inlineStr">
         <is>
-          <t>KODEX 200미국채혼합50</t>
+          <t>TIME 글로벌우주테크&amp;방산액티브</t>
         </is>
       </c>
       <c r="D94" s="33" t="inlineStr">
@@ -7896,39 +7896,39 @@
       </c>
       <c r="E94" s="33" t="inlineStr">
         <is>
-          <t>삼성자산운용(ETF)</t>
+          <t>타임폴리오자산운용</t>
         </is>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
-          <t>2조원</t>
+          <t>2,248억원</t>
         </is>
       </c>
       <c r="G94" s="35" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H94" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I94" s="36" t="n">
-        <v>0.09119999999999999</v>
+        <v>0.0286</v>
       </c>
       <c r="J94" s="36" t="n">
-        <v>0.1365</v>
+        <v>0.2643</v>
       </c>
       <c r="K94" s="37" t="n">
-        <v>-0.2525</v>
+        <v>-0.2932</v>
       </c>
       <c r="L94" s="40" t="n">
-        <v>0.0035</v>
+        <v>0.008</v>
       </c>
       <c r="M94" s="38" t="inlineStr">
         <is>
-          <t>5해 연9.1% · 변동성 13.7% (위험대비 0.46) · 최대낙폭 -25% · 보수 0.35% · 가장 나쁜 창 연9.1%</t>
+          <t>1해 연2.9% · 변동성 26.4% (위험대비 0.00) · 최대낙폭 -29% · 보수 0.80%</t>
         </is>
       </c>
     </row>
@@ -7945,22 +7945,22 @@
       </c>
       <c r="C95" s="14" t="inlineStr">
         <is>
-          <t>TIGER 일본니케이225</t>
+          <t>TIGER 미국투자등급회사채액티브(H)</t>
         </is>
       </c>
       <c r="D95" s="14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>채권형</t>
         </is>
       </c>
       <c r="E95" s="14" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F95" s="28" t="inlineStr">
         <is>
-          <t>3,967억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G95" s="30" t="inlineStr">
@@ -7970,24 +7970,26 @@
       </c>
       <c r="H95" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I95" s="29" t="n">
-        <v>0.1541</v>
+        <v>0.0194</v>
       </c>
       <c r="J95" s="29" t="n">
-        <v>0.2107</v>
+        <v>0.07690000000000001</v>
       </c>
       <c r="K95" s="31" t="n">
-        <v>-0.2394</v>
-      </c>
-      <c r="L95" s="39" t="n">
-        <v>0.0035</v>
+        <v>-0.0713</v>
+      </c>
+      <c r="L95" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M95" s="32" t="inlineStr">
         <is>
-          <t>5해 연15.4% · 변동성 21.1% (위험대비 0.60) · 최대낙폭 -24% · 보수 0.35% · 가장 나쁜 창 연15.4%</t>
+          <t>3해 연1.9% · 변동성 7.7% (위험대비 -0.11) · 최대낙폭 -7% · 가장 나쁜 창 연-2.0%</t>
         </is>
       </c>
     </row>
@@ -8004,22 +8006,22 @@
       </c>
       <c r="C96" s="33" t="inlineStr">
         <is>
-          <t>TIGER 테슬라채권혼합Fn</t>
+          <t>TIGER 미국필라델피아반도체나스닥</t>
         </is>
       </c>
       <c r="D96" s="33" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>반도체&amp;A.I.</t>
         </is>
       </c>
       <c r="E96" s="33" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
-          <t>4,393억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G96" s="35" t="inlineStr">
@@ -8029,24 +8031,26 @@
       </c>
       <c r="H96" s="35" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I96" s="36" t="n">
-        <v>0.0867</v>
+        <v>0.329</v>
       </c>
       <c r="J96" s="36" t="n">
-        <v>0.2019</v>
+        <v>0.3539</v>
       </c>
       <c r="K96" s="37" t="n">
-        <v>-0.2107</v>
-      </c>
-      <c r="L96" s="40" t="n">
-        <v>0.0025</v>
+        <v>-0.3968</v>
+      </c>
+      <c r="L96" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M96" s="38" t="inlineStr">
         <is>
-          <t>3해 연8.7% · 변동성 20.2% (위험대비 0.29) · 최대낙폭 -21% · 보수 0.25% · 가장 나쁜 창 연1.2%</t>
+          <t>5해 연32.9% · 변동성 35.4% (위험대비 0.85) · 최대낙폭 -40% · 가장 나쁜 창 연32.9%</t>
         </is>
       </c>
     </row>
@@ -8063,22 +8067,22 @@
       </c>
       <c r="C97" s="14" t="inlineStr">
         <is>
-          <t>KODEX 인도Nifty50</t>
+          <t>RISE 글로벌원자력</t>
         </is>
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>원자력&amp;전력인프라</t>
         </is>
       </c>
       <c r="E97" s="14" t="inlineStr">
         <is>
-          <t>삼성자산운용(ETF)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F97" s="28" t="inlineStr">
         <is>
-          <t>3,297억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G97" s="30" t="inlineStr">
@@ -8092,20 +8096,22 @@
         </is>
       </c>
       <c r="I97" s="29" t="n">
-        <v>0.0234</v>
+        <v>0.4532</v>
       </c>
       <c r="J97" s="29" t="n">
-        <v>0.1516</v>
+        <v>0.3917</v>
       </c>
       <c r="K97" s="31" t="n">
-        <v>-0.2475</v>
-      </c>
-      <c r="L97" s="39" t="n">
-        <v>0.0019</v>
+        <v>-0.3842</v>
+      </c>
+      <c r="L97" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M97" s="32" t="inlineStr">
         <is>
-          <t>3해 연2.3% · 변동성 15.2% (위험대비 -0.03) · 최대낙폭 -25% · 보수 0.19% · 가장 나쁜 창 연-13.3%</t>
+          <t>3해 연45.3% · 변동성 39.2% (위험대비 1.09) · 최대낙폭 -38% · 가장 나쁜 창 연11.7%</t>
         </is>
       </c>
     </row>
@@ -8122,22 +8128,22 @@
       </c>
       <c r="C98" s="33" t="inlineStr">
         <is>
-          <t>TIGER 미국테크TOP10 INDXX</t>
+          <t>TIGER 차이나반도체FACTSET</t>
         </is>
       </c>
       <c r="D98" s="33" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>중국</t>
         </is>
       </c>
       <c r="E98" s="33" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
-          <t>4조원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G98" s="35" t="inlineStr">
@@ -8147,24 +8153,26 @@
       </c>
       <c r="H98" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I98" s="36" t="n">
-        <v>0.216</v>
+        <v>0.2965</v>
       </c>
       <c r="J98" s="36" t="n">
-        <v>0.2524</v>
+        <v>0.3974</v>
       </c>
       <c r="K98" s="37" t="n">
-        <v>-0.4059</v>
-      </c>
-      <c r="L98" s="40" t="n">
-        <v>0.0049</v>
+        <v>-0.4533</v>
+      </c>
+      <c r="L98" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M98" s="38" t="inlineStr">
         <is>
-          <t>5해 연21.6% · 변동성 25.2% (위험대비 0.74) · 최대낙폭 -41% · 보수 0.49% · 가장 나쁜 창 연15.1%</t>
+          <t>3해 연29.6% · 변동성 39.7% (위험대비 0.68) · 최대낙폭 -45% · 가장 나쁜 창 연29.6%</t>
         </is>
       </c>
     </row>
@@ -8181,22 +8189,22 @@
       </c>
       <c r="C99" s="14" t="inlineStr">
         <is>
-          <t>ACE 미국30년국채액티브(H)</t>
+          <t>TIGER 차이나과창판STAR50(합성)</t>
         </is>
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>중국</t>
         </is>
       </c>
       <c r="E99" s="14" t="inlineStr">
         <is>
-          <t>한국투자신탁운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F99" s="28" t="inlineStr">
         <is>
-          <t>1조원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G99" s="30" t="inlineStr">
@@ -8210,20 +8218,22 @@
         </is>
       </c>
       <c r="I99" s="29" t="n">
-        <v>-0.0398</v>
+        <v>0.2444</v>
       </c>
       <c r="J99" s="29" t="n">
-        <v>0.137</v>
+        <v>0.3654</v>
       </c>
       <c r="K99" s="31" t="n">
-        <v>-0.1731</v>
-      </c>
-      <c r="L99" s="39" t="n">
-        <v>0.0005</v>
+        <v>-0.3919</v>
+      </c>
+      <c r="L99" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M99" s="32" t="inlineStr">
         <is>
-          <t>3해 연-4.0% · 변동성 13.7% (위험대비 -0.50) · 최대낙폭 -17% · 보수 0.05% · 가장 나쁜 창 연-4.0%</t>
+          <t>3해 연24.4% · 변동성 36.5% (위험대비 0.59) · 최대낙폭 -39% · 가장 나쁜 창 연24.4%</t>
         </is>
       </c>
     </row>
@@ -8240,22 +8250,22 @@
       </c>
       <c r="C100" s="33" t="inlineStr">
         <is>
-          <t>TIGER 미국채10년선물</t>
+          <t>ACE 중국과창판STAR50</t>
         </is>
       </c>
       <c r="D100" s="33" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>중국</t>
         </is>
       </c>
       <c r="E100" s="33" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
-          <t>2,171억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G100" s="35" t="inlineStr">
@@ -8265,24 +8275,26 @@
       </c>
       <c r="H100" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I100" s="36" t="n">
-        <v>0.0026</v>
+        <v>0.22</v>
       </c>
       <c r="J100" s="36" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.3696</v>
       </c>
       <c r="K100" s="37" t="n">
-        <v>-0.1589</v>
-      </c>
-      <c r="L100" s="40" t="n">
-        <v>0.0029</v>
+        <v>-0.3923</v>
+      </c>
+      <c r="L100" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M100" s="38" t="inlineStr">
         <is>
-          <t>5해 연0.3% · 변동성 9.7% (위험대비 -0.26) · 최대낙폭 -16% · 보수 0.29% · 가장 나쁜 창 연-3.9%</t>
+          <t>3해 연22.0% · 변동성 37.0% (위험대비 0.52) · 최대낙폭 -39% · 가장 나쁜 창 연22.0%</t>
         </is>
       </c>
     </row>
@@ -8299,49 +8311,51 @@
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>KODEX 미국빅테크10(H)</t>
+          <t>Invesco 원자재</t>
         </is>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>대체</t>
         </is>
       </c>
       <c r="E101" s="14" t="inlineStr">
         <is>
-          <t>삼성자산운용(ETF)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F101" s="28" t="inlineStr">
         <is>
-          <t>6,596억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G101" s="30" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H101" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I101" s="29" t="n">
-        <v>0.1677</v>
+        <v>0.5193</v>
       </c>
       <c r="J101" s="29" t="n">
-        <v>0.2981</v>
+        <v>0.2353</v>
       </c>
       <c r="K101" s="31" t="n">
-        <v>-0.4973</v>
-      </c>
-      <c r="L101" s="39" t="n">
-        <v>0.004500000000000001</v>
+        <v>-0.1529</v>
+      </c>
+      <c r="L101" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M101" s="32" t="inlineStr">
         <is>
-          <t>5해 연16.8% · 변동성 29.8% (위험대비 0.47) · 최대낙폭 -50% · 보수 0.45% · 가장 나쁜 창 연16.1%</t>
+          <t>1해 연51.9% · 변동성 23.5% (위험대비 2.09) · 최대낙폭 -15%</t>
         </is>
       </c>
     </row>
@@ -8358,49 +8372,51 @@
       </c>
       <c r="C102" s="33" t="inlineStr">
         <is>
-          <t>TIGER 미국나스닥바이오</t>
+          <t>Schwab 미국 배당주</t>
         </is>
       </c>
       <c r="D102" s="33" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>주식</t>
         </is>
       </c>
       <c r="E102" s="33" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
-          <t>1,075억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G102" s="35" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H102" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I102" s="36" t="n">
-        <v>0.1018</v>
+        <v>0.2792</v>
       </c>
       <c r="J102" s="36" t="n">
-        <v>0.2281</v>
+        <v>0.1419</v>
       </c>
       <c r="K102" s="37" t="n">
-        <v>-0.3107</v>
-      </c>
-      <c r="L102" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.092</v>
+      </c>
+      <c r="L102" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M102" s="38" t="inlineStr">
         <is>
-          <t>5해 연10.2% · 변동성 22.8% (위험대비 0.32) · 최대낙폭 -31% · 보수 0.30% · 가장 나쁜 창 연10.2%</t>
+          <t>1해 연27.9% · 변동성 14.2% (위험대비 1.77) · 최대낙폭 -9%</t>
         </is>
       </c>
     </row>
@@ -8417,49 +8433,51 @@
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
-          <t>KODEX 차이나CSI300</t>
+          <t>Vanguard 미국 전체시장</t>
         </is>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>주식</t>
         </is>
       </c>
       <c r="E103" s="14" t="inlineStr">
         <is>
-          <t>삼성자산운용(ETF)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F103" s="28" t="inlineStr">
         <is>
-          <t>2,495억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G103" s="30" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H103" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I103" s="29" t="n">
-        <v>0.0269</v>
+        <v>0.1758</v>
       </c>
       <c r="J103" s="29" t="n">
-        <v>0.1868</v>
+        <v>0.1455</v>
       </c>
       <c r="K103" s="31" t="n">
-        <v>-0.3717</v>
-      </c>
-      <c r="L103" s="39" t="n">
-        <v>0.0012</v>
+        <v>-0.1283</v>
+      </c>
+      <c r="L103" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M103" s="32" t="inlineStr">
         <is>
-          <t>5해 연2.7% · 변동성 18.7% (위험대비 -0.01) · 최대낙폭 -37% · 보수 0.12% · 가장 나쁜 창 연2.7%</t>
+          <t>1해 연17.6% · 변동성 14.6% (위험대비 1.02) · 최대낙폭 -13%</t>
         </is>
       </c>
     </row>
@@ -8476,49 +8494,51 @@
       </c>
       <c r="C104" s="33" t="inlineStr">
         <is>
-          <t>ACE 베트남VN30(합성)</t>
+          <t>Vanguard 선진국(미국 제외)</t>
         </is>
       </c>
       <c r="D104" s="33" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>주식</t>
         </is>
       </c>
       <c r="E104" s="33" t="inlineStr">
         <is>
-          <t>한국투신운용(ETF)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F104" s="34" t="inlineStr">
         <is>
-          <t>3,787억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G104" s="35" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H104" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I104" s="36" t="n">
-        <v>0.0707</v>
+        <v>0.2346</v>
       </c>
       <c r="J104" s="36" t="n">
-        <v>0.2053</v>
+        <v>0.1726</v>
       </c>
       <c r="K104" s="37" t="n">
-        <v>-0.423</v>
-      </c>
-      <c r="L104" s="40" t="n">
-        <v>0.006999999999999999</v>
+        <v>-0.1323</v>
+      </c>
+      <c r="L104" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M104" s="38" t="inlineStr">
         <is>
-          <t>5해 연7.1% · 변동성 20.5% (위험대비 0.21) · 최대낙폭 -42% · 보수 0.70% · 가장 나쁜 창 연3.8%</t>
+          <t>1해 연23.5% · 변동성 17.3% (위험대비 1.20) · 최대낙폭 -13%</t>
         </is>
       </c>
     </row>
@@ -8535,49 +8555,51 @@
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>TIGER 차이나CSI300</t>
+          <t>Vanguard 배당성장</t>
         </is>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>주식</t>
         </is>
       </c>
       <c r="E105" s="14" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F105" s="28" t="inlineStr">
         <is>
-          <t>1,275억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G105" s="30" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H105" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I105" s="29" t="n">
-        <v>0.0215</v>
+        <v>0.1239</v>
       </c>
       <c r="J105" s="29" t="n">
-        <v>0.1969</v>
+        <v>0.127</v>
       </c>
       <c r="K105" s="31" t="n">
-        <v>-0.3801</v>
-      </c>
-      <c r="L105" s="39" t="n">
-        <v>0.0063</v>
+        <v>-0.1365</v>
+      </c>
+      <c r="L105" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M105" s="32" t="inlineStr">
         <is>
-          <t>5해 연2.1% · 변동성 19.7% (위험대비 -0.03) · 최대낙폭 -38% · 보수 0.63% · 가장 나쁜 창 연2.1%</t>
+          <t>1해 연12.4% · 변동성 12.7% (위험대비 0.75) · 최대낙폭 -14%</t>
         </is>
       </c>
     </row>
@@ -8594,49 +8616,51 @@
       </c>
       <c r="C106" s="33" t="inlineStr">
         <is>
-          <t>TIGER 미국30년국채스트립액티브(합성 H)</t>
+          <t>iShares 러셀2000 (미국 중소형)</t>
         </is>
       </c>
       <c r="D106" s="33" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>주식</t>
         </is>
       </c>
       <c r="E106" s="33" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
-          <t>3,817억원</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G106" s="35" t="inlineStr">
         <is>
-          <t>다년 실측</t>
+          <t>1해 실측</t>
         </is>
       </c>
       <c r="H106" s="35" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>1해</t>
         </is>
       </c>
       <c r="I106" s="36" t="n">
-        <v>-0.09630000000000001</v>
+        <v>0.2092</v>
       </c>
       <c r="J106" s="36" t="n">
-        <v>0.2278</v>
+        <v>0.1952</v>
       </c>
       <c r="K106" s="37" t="n">
-        <v>-0.3277</v>
-      </c>
-      <c r="L106" s="40" t="n">
-        <v>0.0015</v>
+        <v>-0.171</v>
+      </c>
+      <c r="L106" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M106" s="38" t="inlineStr">
         <is>
-          <t>3해 연-9.6% · 변동성 22.8% (위험대비 -0.55) · 최대낙폭 -33% · 보수 0.15% · 가장 나쁜 창 연-9.6%</t>
+          <t>1해 연20.9% · 변동성 19.5% (위험대비 0.93) · 최대낙폭 -17%</t>
         </is>
       </c>
     </row>
@@ -12567,11 +12591,11 @@
         </is>
       </c>
       <c r="B29" s="39" t="n">
-        <v>0.0621</v>
+        <v>0.0561</v>
       </c>
       <c r="C29" s="45" t="inlineStr">
         <is>
-          <t>해외주식 60% · 해외채권 40%</t>
+          <t>해외주식 40% · 해외채권 40% · 대체 20%</t>
         </is>
       </c>
       <c r="D29" s="46" t="n"/>

</xml_diff>

<commit_message>
data(proposal): 해외 ETF 일봉 수집 (2026-09-20 05:47)
</commit_message>
<xml_diff>
--- a/고객제안서_자산배분.xlsx
+++ b/고객제안서_자산배분.xlsx
@@ -1376,7 +1376,7 @@
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>유니버스 2026-09-20 14:35:38 · 문서 2026-09-20 14:35 (KST)</t>
+          <t>유니버스 2026-09-20 14:47:28 · 문서 2026-09-20 14:47 (KST)</t>
         </is>
       </c>
     </row>
@@ -2392,10 +2392,10 @@
         <v>0.1747404299625906</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.1769</v>
+        <v>0.1834939037658289</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>-0.2640451703972575</v>
+        <v>-0.3371736857143508</v>
       </c>
     </row>
     <row r="11">
@@ -7237,7 +7237,7 @@
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>ACE 미국나스닥100미국채혼합50액티브</t>
+          <t>ACE 미국배당다우존스</t>
         </is>
       </c>
       <c r="D83" s="14" t="inlineStr">
@@ -7247,12 +7247,12 @@
       </c>
       <c r="E83" s="14" t="inlineStr">
         <is>
-          <t>한국투자신탁운용</t>
+          <t>한국투신운용(ETF)</t>
         </is>
       </c>
       <c r="F83" s="28" t="inlineStr">
         <is>
-          <t>9,455억원</t>
+          <t>9,703억원</t>
         </is>
       </c>
       <c r="G83" s="30" t="inlineStr">
@@ -7266,20 +7266,20 @@
         </is>
       </c>
       <c r="I83" s="29" t="n">
-        <v>0.1323</v>
+        <v>0.1576</v>
       </c>
       <c r="J83" s="29" t="n">
-        <v>0.09820000000000001</v>
+        <v>0.1409</v>
       </c>
       <c r="K83" s="31" t="n">
-        <v>-0.1486</v>
+        <v>-0.1321</v>
       </c>
       <c r="L83" s="39" t="n">
-        <v>0.0015</v>
+        <v>0.0001</v>
       </c>
       <c r="M83" s="32" t="inlineStr">
         <is>
-          <t>3해 연13.2% · 변동성 9.8% (위험대비 1.06) · 최대낙폭 -15% · 보수 0.15% · 가장 나쁜 창 연11.6%</t>
+          <t>3해 연15.8% · 변동성 14.1% (위험대비 0.92) · 최대낙폭 -13% · 보수 0.01% · 가장 나쁜 창 연15.8%</t>
         </is>
       </c>
     </row>
@@ -7296,7 +7296,7 @@
       </c>
       <c r="C84" s="33" t="inlineStr">
         <is>
-          <t>SOL 미국S&amp;P500</t>
+          <t>ACE 미국나스닥100미국채혼합50액티브</t>
         </is>
       </c>
       <c r="D84" s="33" t="inlineStr">
@@ -7306,12 +7306,12 @@
       </c>
       <c r="E84" s="33" t="inlineStr">
         <is>
-          <t>신한자산운용</t>
+          <t>한국투자신탁운용</t>
         </is>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
-          <t>2,987억원</t>
+          <t>9,455억원</t>
         </is>
       </c>
       <c r="G84" s="35" t="inlineStr">
@@ -7325,20 +7325,20 @@
         </is>
       </c>
       <c r="I84" s="36" t="n">
-        <v>0.2146</v>
+        <v>0.1323</v>
       </c>
       <c r="J84" s="36" t="n">
-        <v>0.1556</v>
+        <v>0.09820000000000001</v>
       </c>
       <c r="K84" s="37" t="n">
-        <v>-0.1924</v>
+        <v>-0.1486</v>
       </c>
       <c r="L84" s="40" t="n">
-        <v>4.7e-05</v>
+        <v>0.0015</v>
       </c>
       <c r="M84" s="38" t="inlineStr">
         <is>
-          <t>3해 연21.5% · 변동성 15.6% (위험대비 1.20) · 최대낙폭 -19% · 보수 0.00% · 가장 나쁜 창 연16.8%</t>
+          <t>3해 연13.2% · 변동성 9.8% (위험대비 1.06) · 최대낙폭 -15% · 보수 0.15% · 가장 나쁜 창 연11.6%</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="C85" s="14" t="inlineStr">
         <is>
-          <t>SOL 미국TOP5채권혼합50</t>
+          <t>SOL 미국S&amp;P500</t>
         </is>
       </c>
       <c r="D85" s="14" t="inlineStr">
@@ -7370,7 +7370,7 @@
       </c>
       <c r="F85" s="28" t="inlineStr">
         <is>
-          <t>1,248억원</t>
+          <t>2,987억원</t>
         </is>
       </c>
       <c r="G85" s="30" t="inlineStr">
@@ -7384,20 +7384,20 @@
         </is>
       </c>
       <c r="I85" s="29" t="n">
-        <v>0.1197</v>
+        <v>0.2146</v>
       </c>
       <c r="J85" s="29" t="n">
-        <v>0.098</v>
+        <v>0.1556</v>
       </c>
       <c r="K85" s="31" t="n">
-        <v>-0.113</v>
+        <v>-0.1924</v>
       </c>
       <c r="L85" s="39" t="n">
-        <v>0.0025</v>
+        <v>4.7e-05</v>
       </c>
       <c r="M85" s="32" t="inlineStr">
         <is>
-          <t>3해 연12.0% · 변동성 9.8% (위험대비 0.93) · 최대낙폭 -11% · 보수 0.25% · 가장 나쁜 창 연11.9%</t>
+          <t>3해 연21.5% · 변동성 15.6% (위험대비 1.20) · 최대낙폭 -19% · 보수 0.00% · 가장 나쁜 창 연16.8%</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C86" s="33" t="inlineStr">
         <is>
-          <t>ACE 미국배당다우존스</t>
+          <t>SOL 미국TOP5채권혼합50</t>
         </is>
       </c>
       <c r="D86" s="33" t="inlineStr">
@@ -7424,12 +7424,12 @@
       </c>
       <c r="E86" s="33" t="inlineStr">
         <is>
-          <t>한국투신운용(ETF)</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
-          <t>9,703억원</t>
+          <t>1,248억원</t>
         </is>
       </c>
       <c r="G86" s="35" t="inlineStr">
@@ -7443,20 +7443,20 @@
         </is>
       </c>
       <c r="I86" s="36" t="n">
-        <v>0.1576</v>
+        <v>0.1197</v>
       </c>
       <c r="J86" s="36" t="n">
-        <v>0.1409</v>
+        <v>0.098</v>
       </c>
       <c r="K86" s="37" t="n">
-        <v>-0.1321</v>
+        <v>-0.113</v>
       </c>
       <c r="L86" s="40" t="n">
-        <v>0.0001</v>
+        <v>0.0025</v>
       </c>
       <c r="M86" s="38" t="inlineStr">
         <is>
-          <t>3해 연15.8% · 변동성 14.1% (위험대비 0.92) · 최대낙폭 -13% · 보수 0.01% · 가장 나쁜 창 연15.8%</t>
+          <t>3해 연12.0% · 변동성 9.8% (위험대비 0.93) · 최대낙폭 -11% · 보수 0.25% · 가장 나쁜 창 연11.9%</t>
         </is>
       </c>
     </row>
@@ -7945,12 +7945,12 @@
       </c>
       <c r="C95" s="14" t="inlineStr">
         <is>
-          <t>TIGER 미국투자등급회사채액티브(H)</t>
+          <t>SPDR 금</t>
         </is>
       </c>
       <c r="D95" s="14" t="inlineStr">
         <is>
-          <t>채권형</t>
+          <t>대체</t>
         </is>
       </c>
       <c r="E95" s="14" t="inlineStr">
@@ -7970,17 +7970,17 @@
       </c>
       <c r="H95" s="30" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I95" s="29" t="n">
-        <v>0.0194</v>
+        <v>0.2325</v>
       </c>
       <c r="J95" s="29" t="n">
-        <v>0.07690000000000001</v>
+        <v>0.2006</v>
       </c>
       <c r="K95" s="31" t="n">
-        <v>-0.0713</v>
+        <v>-0.2618</v>
       </c>
       <c r="L95" s="28" t="inlineStr">
         <is>
@@ -7989,7 +7989,7 @@
       </c>
       <c r="M95" s="32" t="inlineStr">
         <is>
-          <t>3해 연1.9% · 변동성 7.7% (위험대비 -0.11) · 최대낙폭 -7% · 가장 나쁜 창 연-2.0%</t>
+          <t>5해 연23.2% · 변동성 20.1% (위험대비 1.02) · 최대낙폭 -26% · 가장 나쁜 창 연19.8%</t>
         </is>
       </c>
     </row>
@@ -8006,12 +8006,12 @@
       </c>
       <c r="C96" s="33" t="inlineStr">
         <is>
-          <t>TIGER 미국필라델피아반도체나스닥</t>
+          <t>Invesco 원자재</t>
         </is>
       </c>
       <c r="D96" s="33" t="inlineStr">
         <is>
-          <t>반도체&amp;A.I.</t>
+          <t>대체</t>
         </is>
       </c>
       <c r="E96" s="33" t="inlineStr">
@@ -8035,13 +8035,13 @@
         </is>
       </c>
       <c r="I96" s="36" t="n">
-        <v>0.329</v>
+        <v>0.1838</v>
       </c>
       <c r="J96" s="36" t="n">
-        <v>0.3539</v>
+        <v>0.2098</v>
       </c>
       <c r="K96" s="37" t="n">
-        <v>-0.3968</v>
+        <v>-0.25</v>
       </c>
       <c r="L96" s="34" t="inlineStr">
         <is>
@@ -8050,7 +8050,7 @@
       </c>
       <c r="M96" s="38" t="inlineStr">
         <is>
-          <t>5해 연32.9% · 변동성 35.4% (위험대비 0.85) · 최대낙폭 -40% · 가장 나쁜 창 연32.9%</t>
+          <t>5해 연18.4% · 변동성 21.0% (위험대비 0.74) · 최대낙폭 -25% · 가장 나쁜 창 연15.7%</t>
         </is>
       </c>
     </row>
@@ -8067,12 +8067,12 @@
       </c>
       <c r="C97" s="14" t="inlineStr">
         <is>
-          <t>RISE 글로벌원자력</t>
+          <t>iShares 미국채 1-3년</t>
         </is>
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>원자력&amp;전력인프라</t>
+          <t>채권</t>
         </is>
       </c>
       <c r="E97" s="14" t="inlineStr">
@@ -8092,17 +8092,17 @@
       </c>
       <c r="H97" s="30" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I97" s="29" t="n">
-        <v>0.4532</v>
+        <v>0.05309999999999999</v>
       </c>
       <c r="J97" s="29" t="n">
-        <v>0.3917</v>
+        <v>0.0968</v>
       </c>
       <c r="K97" s="31" t="n">
-        <v>-0.3842</v>
+        <v>-0.1396</v>
       </c>
       <c r="L97" s="28" t="inlineStr">
         <is>
@@ -8111,7 +8111,7 @@
       </c>
       <c r="M97" s="32" t="inlineStr">
         <is>
-          <t>3해 연45.3% · 변동성 39.2% (위험대비 1.09) · 최대낙폭 -38% · 가장 나쁜 창 연11.7%</t>
+          <t>5해 연5.3% · 변동성 9.7% (위험대비 0.26) · 최대낙폭 -14% · 가장 나쁜 창 연2.2%</t>
         </is>
       </c>
     </row>
@@ -8128,12 +8128,12 @@
       </c>
       <c r="C98" s="33" t="inlineStr">
         <is>
-          <t>TIGER 차이나반도체FACTSET</t>
+          <t>iShares 하이일드 회사채</t>
         </is>
       </c>
       <c r="D98" s="33" t="inlineStr">
         <is>
-          <t>중국</t>
+          <t>채권</t>
         </is>
       </c>
       <c r="E98" s="33" t="inlineStr">
@@ -8153,17 +8153,17 @@
       </c>
       <c r="H98" s="35" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I98" s="36" t="n">
-        <v>0.2965</v>
+        <v>0.0709</v>
       </c>
       <c r="J98" s="36" t="n">
-        <v>0.3974</v>
+        <v>0.1136</v>
       </c>
       <c r="K98" s="37" t="n">
-        <v>-0.4533</v>
+        <v>-0.1402</v>
       </c>
       <c r="L98" s="34" t="inlineStr">
         <is>
@@ -8172,7 +8172,7 @@
       </c>
       <c r="M98" s="38" t="inlineStr">
         <is>
-          <t>3해 연29.6% · 변동성 39.7% (위험대비 0.68) · 최대낙폭 -45% · 가장 나쁜 창 연29.6%</t>
+          <t>5해 연7.1% · 변동성 11.4% (위험대비 0.38) · 최대낙폭 -14% · 가장 나쁜 창 연3.5%</t>
         </is>
       </c>
     </row>
@@ -8189,12 +8189,12 @@
       </c>
       <c r="C99" s="14" t="inlineStr">
         <is>
-          <t>TIGER 차이나과창판STAR50(합성)</t>
+          <t>TIGER 미국투자등급회사채액티브(H)</t>
         </is>
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>중국</t>
+          <t>채권형</t>
         </is>
       </c>
       <c r="E99" s="14" t="inlineStr">
@@ -8218,13 +8218,13 @@
         </is>
       </c>
       <c r="I99" s="29" t="n">
-        <v>0.2444</v>
+        <v>0.0194</v>
       </c>
       <c r="J99" s="29" t="n">
-        <v>0.3654</v>
+        <v>0.07690000000000001</v>
       </c>
       <c r="K99" s="31" t="n">
-        <v>-0.3919</v>
+        <v>-0.0713</v>
       </c>
       <c r="L99" s="28" t="inlineStr">
         <is>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="M99" s="32" t="inlineStr">
         <is>
-          <t>3해 연24.4% · 변동성 36.5% (위험대비 0.59) · 최대낙폭 -39% · 가장 나쁜 창 연24.4%</t>
+          <t>3해 연1.9% · 변동성 7.7% (위험대비 -0.11) · 최대낙폭 -7% · 가장 나쁜 창 연-2.0%</t>
         </is>
       </c>
     </row>
@@ -8250,12 +8250,12 @@
       </c>
       <c r="C100" s="33" t="inlineStr">
         <is>
-          <t>ACE 중국과창판STAR50</t>
+          <t>Vanguard 배당성장</t>
         </is>
       </c>
       <c r="D100" s="33" t="inlineStr">
         <is>
-          <t>중국</t>
+          <t>주식</t>
         </is>
       </c>
       <c r="E100" s="33" t="inlineStr">
@@ -8275,17 +8275,17 @@
       </c>
       <c r="H100" s="35" t="inlineStr">
         <is>
-          <t>3해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I100" s="36" t="n">
-        <v>0.22</v>
+        <v>0.1402</v>
       </c>
       <c r="J100" s="36" t="n">
-        <v>0.3696</v>
+        <v>0.1641</v>
       </c>
       <c r="K100" s="37" t="n">
-        <v>-0.3923</v>
+        <v>-0.1365</v>
       </c>
       <c r="L100" s="34" t="inlineStr">
         <is>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="M100" s="38" t="inlineStr">
         <is>
-          <t>3해 연22.0% · 변동성 37.0% (위험대비 0.52) · 최대낙폭 -39% · 가장 나쁜 창 연22.0%</t>
+          <t>5해 연14.0% · 변동성 16.4% (위험대비 0.68) · 최대낙폭 -14% · 가장 나쁜 창 연12.4%</t>
         </is>
       </c>
     </row>
@@ -8311,12 +8311,12 @@
       </c>
       <c r="C101" s="14" t="inlineStr">
         <is>
-          <t>Invesco 원자재</t>
+          <t>Schwab 미국 배당주</t>
         </is>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>대체</t>
+          <t>주식</t>
         </is>
       </c>
       <c r="E101" s="14" t="inlineStr">
@@ -8331,22 +8331,22 @@
       </c>
       <c r="G101" s="30" t="inlineStr">
         <is>
-          <t>1해 실측</t>
+          <t>다년 실측</t>
         </is>
       </c>
       <c r="H101" s="30" t="inlineStr">
         <is>
-          <t>1해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I101" s="29" t="n">
-        <v>0.5193</v>
+        <v>0.1353</v>
       </c>
       <c r="J101" s="29" t="n">
-        <v>0.2353</v>
+        <v>0.1663</v>
       </c>
       <c r="K101" s="31" t="n">
-        <v>-0.1529</v>
+        <v>-0.1455</v>
       </c>
       <c r="L101" s="28" t="inlineStr">
         <is>
@@ -8355,7 +8355,7 @@
       </c>
       <c r="M101" s="32" t="inlineStr">
         <is>
-          <t>1해 연51.9% · 변동성 23.5% (위험대비 2.09) · 최대낙폭 -15%</t>
+          <t>5해 연13.5% · 변동성 16.6% (위험대비 0.64) · 최대낙폭 -15% · 가장 나쁜 창 연13.5%</t>
         </is>
       </c>
     </row>
@@ -8372,7 +8372,7 @@
       </c>
       <c r="C102" s="33" t="inlineStr">
         <is>
-          <t>Schwab 미국 배당주</t>
+          <t>Vanguard 미국 전체시장</t>
         </is>
       </c>
       <c r="D102" s="33" t="inlineStr">
@@ -8392,22 +8392,22 @@
       </c>
       <c r="G102" s="35" t="inlineStr">
         <is>
-          <t>1해 실측</t>
+          <t>다년 실측</t>
         </is>
       </c>
       <c r="H102" s="35" t="inlineStr">
         <is>
-          <t>1해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I102" s="36" t="n">
-        <v>0.2792</v>
+        <v>0.1574</v>
       </c>
       <c r="J102" s="36" t="n">
-        <v>0.1419</v>
+        <v>0.1895</v>
       </c>
       <c r="K102" s="37" t="n">
-        <v>-0.092</v>
+        <v>-0.1826</v>
       </c>
       <c r="L102" s="34" t="inlineStr">
         <is>
@@ -8416,7 +8416,7 @@
       </c>
       <c r="M102" s="38" t="inlineStr">
         <is>
-          <t>1해 연27.9% · 변동성 14.2% (위험대비 1.77) · 최대낙폭 -9%</t>
+          <t>5해 연15.7% · 변동성 18.9% (위험대비 0.68) · 최대낙폭 -18% · 가장 나쁜 창 연15.7%</t>
         </is>
       </c>
     </row>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
-          <t>Vanguard 미국 전체시장</t>
+          <t>Vanguard 선진국(미국 제외)</t>
         </is>
       </c>
       <c r="D103" s="14" t="inlineStr">
@@ -8453,22 +8453,22 @@
       </c>
       <c r="G103" s="30" t="inlineStr">
         <is>
-          <t>1해 실측</t>
+          <t>다년 실측</t>
         </is>
       </c>
       <c r="H103" s="30" t="inlineStr">
         <is>
-          <t>1해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I103" s="29" t="n">
-        <v>0.1758</v>
+        <v>0.1349</v>
       </c>
       <c r="J103" s="29" t="n">
-        <v>0.1455</v>
+        <v>0.1707</v>
       </c>
       <c r="K103" s="31" t="n">
-        <v>-0.1283</v>
+        <v>-0.1538</v>
       </c>
       <c r="L103" s="28" t="inlineStr">
         <is>
@@ -8477,7 +8477,7 @@
       </c>
       <c r="M103" s="32" t="inlineStr">
         <is>
-          <t>1해 연17.6% · 변동성 14.6% (위험대비 1.02) · 최대낙폭 -13%</t>
+          <t>5해 연13.5% · 변동성 17.1% (위험대비 0.63) · 최대낙폭 -15% · 가장 나쁜 창 연13.5%</t>
         </is>
       </c>
     </row>
@@ -8494,12 +8494,12 @@
       </c>
       <c r="C104" s="33" t="inlineStr">
         <is>
-          <t>Vanguard 선진국(미국 제외)</t>
+          <t>iShares 미국 종합채권</t>
         </is>
       </c>
       <c r="D104" s="33" t="inlineStr">
         <is>
-          <t>주식</t>
+          <t>채권</t>
         </is>
       </c>
       <c r="E104" s="33" t="inlineStr">
@@ -8514,22 +8514,22 @@
       </c>
       <c r="G104" s="35" t="inlineStr">
         <is>
-          <t>1해 실측</t>
+          <t>다년 실측</t>
         </is>
       </c>
       <c r="H104" s="35" t="inlineStr">
         <is>
-          <t>1해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I104" s="36" t="n">
-        <v>0.2346</v>
+        <v>0.0301</v>
       </c>
       <c r="J104" s="36" t="n">
-        <v>0.1726</v>
+        <v>0.1102</v>
       </c>
       <c r="K104" s="37" t="n">
-        <v>-0.1323</v>
+        <v>-0.1544</v>
       </c>
       <c r="L104" s="34" t="inlineStr">
         <is>
@@ -8538,7 +8538,7 @@
       </c>
       <c r="M104" s="38" t="inlineStr">
         <is>
-          <t>1해 연23.5% · 변동성 17.3% (위험대비 1.20) · 최대낙폭 -13%</t>
+          <t>5해 연3.0% · 변동성 11.0% (위험대비 0.02) · 최대낙폭 -15% · 가장 나쁜 창 연-0.0%</t>
         </is>
       </c>
     </row>
@@ -8555,12 +8555,12 @@
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>Vanguard 배당성장</t>
+          <t>TIGER 미국필라델피아반도체나스닥</t>
         </is>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>주식</t>
+          <t>반도체&amp;A.I.</t>
         </is>
       </c>
       <c r="E105" s="14" t="inlineStr">
@@ -8575,22 +8575,22 @@
       </c>
       <c r="G105" s="30" t="inlineStr">
         <is>
-          <t>1해 실측</t>
+          <t>다년 실측</t>
         </is>
       </c>
       <c r="H105" s="30" t="inlineStr">
         <is>
-          <t>1해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I105" s="29" t="n">
-        <v>0.1239</v>
+        <v>0.329</v>
       </c>
       <c r="J105" s="29" t="n">
-        <v>0.127</v>
+        <v>0.3539</v>
       </c>
       <c r="K105" s="31" t="n">
-        <v>-0.1365</v>
+        <v>-0.3968</v>
       </c>
       <c r="L105" s="28" t="inlineStr">
         <is>
@@ -8599,7 +8599,7 @@
       </c>
       <c r="M105" s="32" t="inlineStr">
         <is>
-          <t>1해 연12.4% · 변동성 12.7% (위험대비 0.75) · 최대낙폭 -14%</t>
+          <t>5해 연32.9% · 변동성 35.4% (위험대비 0.85) · 최대낙폭 -40% · 가장 나쁜 창 연32.9%</t>
         </is>
       </c>
     </row>
@@ -8616,7 +8616,7 @@
       </c>
       <c r="C106" s="33" t="inlineStr">
         <is>
-          <t>iShares 러셀2000 (미국 중소형)</t>
+          <t>Vanguard 신흥국</t>
         </is>
       </c>
       <c r="D106" s="33" t="inlineStr">
@@ -8636,22 +8636,22 @@
       </c>
       <c r="G106" s="35" t="inlineStr">
         <is>
-          <t>1해 실측</t>
+          <t>다년 실측</t>
         </is>
       </c>
       <c r="H106" s="35" t="inlineStr">
         <is>
-          <t>1해</t>
+          <t>5해</t>
         </is>
       </c>
       <c r="I106" s="36" t="n">
-        <v>0.2092</v>
+        <v>0.09710000000000001</v>
       </c>
       <c r="J106" s="36" t="n">
-        <v>0.1952</v>
+        <v>0.1743</v>
       </c>
       <c r="K106" s="37" t="n">
-        <v>-0.171</v>
+        <v>-0.1624</v>
       </c>
       <c r="L106" s="34" t="inlineStr">
         <is>
@@ -8660,7 +8660,7 @@
       </c>
       <c r="M106" s="38" t="inlineStr">
         <is>
-          <t>1해 연20.9% · 변동성 19.5% (위험대비 0.93) · 최대낙폭 -17%</t>
+          <t>5해 연9.7% · 변동성 17.4% (위험대비 0.40) · 최대낙폭 -16% · 가장 나쁜 창 연9.7%</t>
         </is>
       </c>
     </row>
@@ -12194,7 +12194,7 @@
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="E9" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
data(proposal): 펀드 기준가 계열 수집 (2026-09-20 07:00)
</commit_message>
<xml_diff>
--- a/고객제안서_자산배분.xlsx
+++ b/고객제안서_자산배분.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제안서" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="배분규칙" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자산군" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상품" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기대수익률" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="제안서" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="배분규칙" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="자산군" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="상품" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="출처" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="기대수익률" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="사용법" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'상품'!$A$6:$M$156</definedName>
@@ -1078,7 +1078,7 @@
         <v/>
       </c>
       <c r="G23" s="17" t="n">
-        <v>0.0553</v>
+        <v>0.0535</v>
       </c>
       <c r="H23" s="15">
         <f>IF(ISNUMBER($F23),$F23,0)</f>
@@ -1376,7 +1376,7 @@
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>유니버스 2026-09-20 15:44:21 · 문서 2026-09-20 15:44 (KST)</t>
+          <t>유니버스 2026-09-20 16:00:00 · 문서 2026-09-20 16:00 (KST)</t>
         </is>
       </c>
     </row>
@@ -2366,12 +2366,10 @@
         <v>0.333284</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.168402030225</v>
-      </c>
-      <c r="F9" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.18285</v>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>-0.1577</v>
       </c>
     </row>
     <row r="10">
@@ -2409,13 +2407,13 @@
         <v>99</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>0.1049382716049381</v>
+        <v>0.09780242562454644</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.2923973274425171</v>
+        <v>0.2921539773352639</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>-0.3235610824922673</v>
+        <v>-0.3237114148035969</v>
       </c>
     </row>
     <row r="12">
@@ -2434,12 +2432,10 @@
         <v>0.1178985</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.132657723045</v>
-      </c>
-      <c r="F12" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1361</v>
+      </c>
+      <c r="F12" s="29" t="n">
+        <v>-0.11885</v>
       </c>
     </row>
     <row r="13">
@@ -2458,12 +2454,10 @@
         <v>0.028086</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.000591987885</v>
-      </c>
-      <c r="F13" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0326</v>
+      </c>
+      <c r="F13" s="29" t="n">
+        <v>-0.0344</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -4407,7 +4401,7 @@
       </c>
       <c r="F36" s="34" t="inlineStr">
         <is>
-          <t>932조원</t>
+          <t>931조원</t>
         </is>
       </c>
       <c r="G36" s="35" t="inlineStr">
@@ -4529,7 +4523,7 @@
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
-          <t>902조원</t>
+          <t>901조원</t>
         </is>
       </c>
       <c r="G38" s="35" t="inlineStr">
@@ -4651,7 +4645,7 @@
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
-          <t>1,288조원</t>
+          <t>1,287조원</t>
         </is>
       </c>
       <c r="G40" s="35" t="inlineStr">
@@ -4712,7 +4706,7 @@
       </c>
       <c r="F41" s="28" t="inlineStr">
         <is>
-          <t>570조원</t>
+          <t>569조원</t>
         </is>
       </c>
       <c r="G41" s="30" t="inlineStr">
@@ -4834,7 +4828,7 @@
       </c>
       <c r="F43" s="28" t="inlineStr">
         <is>
-          <t>1,512조원</t>
+          <t>1,511조원</t>
         </is>
       </c>
       <c r="G43" s="30" t="inlineStr">
@@ -5078,7 +5072,7 @@
       </c>
       <c r="F47" s="28" t="inlineStr">
         <is>
-          <t>1,425조원</t>
+          <t>1,424조원</t>
         </is>
       </c>
       <c r="G47" s="30" t="inlineStr">
@@ -5139,7 +5133,7 @@
       </c>
       <c r="F48" s="34" t="inlineStr">
         <is>
-          <t>1,177조원</t>
+          <t>1,176조원</t>
         </is>
       </c>
       <c r="G48" s="35" t="inlineStr">
@@ -5444,7 +5438,7 @@
       </c>
       <c r="F53" s="28" t="inlineStr">
         <is>
-          <t>6,799조원</t>
+          <t>6,794조원</t>
         </is>
       </c>
       <c r="G53" s="30" t="inlineStr">
@@ -5505,7 +5499,7 @@
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
-          <t>179조원</t>
+          <t>178조원</t>
         </is>
       </c>
       <c r="G54" s="35" t="inlineStr">
@@ -8673,22 +8667,22 @@
       </c>
       <c r="C107" s="14" t="inlineStr">
         <is>
-          <t>대신우량단기채증권투자신탁3[채권](운용)</t>
+          <t>이지스코어리테일부동산투자신탁 126</t>
         </is>
       </c>
       <c r="D107" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내대체</t>
         </is>
       </c>
       <c r="E107" s="14" t="inlineStr">
         <is>
-          <t>대신자산운용</t>
+          <t>이지스자산운용</t>
         </is>
       </c>
       <c r="F107" s="28" t="inlineStr">
         <is>
-          <t>192억원</t>
+          <t>606억원</t>
         </is>
       </c>
       <c r="G107" s="30" t="inlineStr">
@@ -8698,28 +8692,26 @@
       </c>
       <c r="H107" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I107" s="29" t="n">
-        <v>0.0363</v>
+        <v>0.0469</v>
       </c>
       <c r="J107" s="29" t="n">
-        <v>0.0012</v>
-      </c>
-      <c r="K107" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0069</v>
+      </c>
+      <c r="K107" s="31" t="n">
+        <v>0</v>
       </c>
       <c r="L107" s="28" t="inlineStr">
         <is>
-          <t>0.06~0.26%</t>
+          <t>0.00~0.00%</t>
         </is>
       </c>
       <c r="M107" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.6% · 변동성 0.1% (위험대비 6.83) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.06% · 가장 나쁜 창 연3.2%</t>
+          <t>3해 연4.7% · 변동성 0.7% (위험대비 2.72) (달 간격) · 최대낙폭 0% · 보수 0.00% · 가장 나쁜 창 연4.7%</t>
         </is>
       </c>
     </row>
@@ -8736,22 +8728,22 @@
       </c>
       <c r="C108" s="33" t="inlineStr">
         <is>
-          <t>KB내일드림초단기채증권투자신탁(채권)(운용)</t>
+          <t>이지스리테일부동산투자신탁299</t>
         </is>
       </c>
       <c r="D108" s="33" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내대체</t>
         </is>
       </c>
       <c r="E108" s="33" t="inlineStr">
         <is>
-          <t>케이비자산운용</t>
+          <t>이지스자산운용</t>
         </is>
       </c>
       <c r="F108" s="34" t="inlineStr">
         <is>
-          <t>2조원</t>
+          <t>211억원</t>
         </is>
       </c>
       <c r="G108" s="35" t="inlineStr">
@@ -8765,24 +8757,20 @@
         </is>
       </c>
       <c r="I108" s="36" t="n">
-        <v>0.0362</v>
+        <v>0.0398</v>
       </c>
       <c r="J108" s="36" t="n">
-        <v>0.0011</v>
-      </c>
-      <c r="K108" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L108" s="34" t="inlineStr">
-        <is>
-          <t>0.09~0.23%</t>
-        </is>
+        <v>0.0212</v>
+      </c>
+      <c r="K108" s="37" t="n">
+        <v>-0.0241</v>
+      </c>
+      <c r="L108" s="40" t="n">
+        <v>0.0006400000000000001</v>
       </c>
       <c r="M108" s="38" t="inlineStr">
         <is>
-          <t>3해 연3.6% · 변동성 0.1% (위험대비 7.36) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.09% · 가장 나쁜 창 연3.1%</t>
+          <t>3해 연4.0% · 변동성 2.1% (위험대비 0.55) (달 간격) · 최대낙폭 -2% · 보수 0.06% · 가장 나쁜 창 연4.0%</t>
         </is>
       </c>
     </row>
@@ -8799,12 +8787,12 @@
       </c>
       <c r="C109" s="14" t="inlineStr">
         <is>
-          <t>마이다스초단기채프리미엄증권투자신탁(채권)(운용)</t>
+          <t>마이다스거북이90증권자투자신탁 1(주식)(운용)</t>
         </is>
       </c>
       <c r="D109" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내대체</t>
         </is>
       </c>
       <c r="E109" s="14" t="inlineStr">
@@ -8814,7 +8802,7 @@
       </c>
       <c r="F109" s="28" t="inlineStr">
         <is>
-          <t>5,025억원</t>
+          <t>1,952억원</t>
         </is>
       </c>
       <c r="G109" s="30" t="inlineStr">
@@ -8824,28 +8812,26 @@
       </c>
       <c r="H109" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I109" s="29" t="n">
-        <v>0.0343</v>
+        <v>0.1644</v>
       </c>
       <c r="J109" s="29" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="K109" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0808</v>
+      </c>
+      <c r="K109" s="31" t="n">
+        <v>-0.0366</v>
       </c>
       <c r="L109" s="28" t="inlineStr">
         <is>
-          <t>0.10~0.40%</t>
+          <t>0.59~2.09%</t>
         </is>
       </c>
       <c r="M109" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.4% · 변동성 0.1% (위험대비 6.20) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.10% · 가장 나쁜 창 연3.4%</t>
+          <t>3해 연16.4% · 변동성 8.1% (위험대비 1.69) (달 간격) · 최대낙폭 -4% · 보수 0.59% · 가장 나쁜 창 연16.4%</t>
         </is>
       </c>
     </row>
@@ -8862,7 +8848,7 @@
       </c>
       <c r="C110" s="33" t="inlineStr">
         <is>
-          <t>코레이트초단기금리혼합자산투자신탁_운용</t>
+          <t>유진챔피언중단기채증권자투자신탁(채권)</t>
         </is>
       </c>
       <c r="D110" s="33" t="inlineStr">
@@ -8872,12 +8858,12 @@
       </c>
       <c r="E110" s="33" t="inlineStr">
         <is>
-          <t>코레이트자산운용</t>
+          <t>유진자산운용</t>
         </is>
       </c>
       <c r="F110" s="34" t="inlineStr">
         <is>
-          <t>9,418억원</t>
+          <t>1,392억원</t>
         </is>
       </c>
       <c r="G110" s="35" t="inlineStr">
@@ -8891,24 +8877,22 @@
         </is>
       </c>
       <c r="I110" s="36" t="n">
-        <v>0.0371</v>
+        <v>0.0073</v>
       </c>
       <c r="J110" s="36" t="n">
-        <v>0.0008</v>
-      </c>
-      <c r="K110" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.035</v>
+      </c>
+      <c r="K110" s="37" t="n">
+        <v>-0.04</v>
       </c>
       <c r="L110" s="34" t="inlineStr">
         <is>
-          <t>0.11~0.27%</t>
+          <t>0.11~0.41%</t>
         </is>
       </c>
       <c r="M110" s="38" t="inlineStr">
         <is>
-          <t>3해 연3.7% · 변동성 0.1% (위험대비 11.25) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.11% · 가장 나쁜 창 연3.3%</t>
+          <t>3해 연0.7% · 변동성 3.5% (위험대비 -0.59) (달 간격) · 최대낙폭 -4% · 보수 0.11% · 가장 나쁜 창 연-0.1%</t>
         </is>
       </c>
     </row>
@@ -8925,22 +8909,22 @@
       </c>
       <c r="C111" s="14" t="inlineStr">
         <is>
-          <t>BNK내일환매초단기채증권자투자신탁(채권)</t>
+          <t>우리반도체BIG2플러스증권투자신탁(채권혼합)</t>
         </is>
       </c>
       <c r="D111" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내혼합형</t>
         </is>
       </c>
       <c r="E111" s="14" t="inlineStr">
         <is>
-          <t>비엔케이자산운용</t>
+          <t>우리자산운용</t>
         </is>
       </c>
       <c r="F111" s="28" t="inlineStr">
         <is>
-          <t>182억원</t>
+          <t>4,207억원</t>
         </is>
       </c>
       <c r="G111" s="30" t="inlineStr">
@@ -8950,28 +8934,26 @@
       </c>
       <c r="H111" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I111" s="29" t="n">
-        <v>0.0326</v>
+        <v>0.2141</v>
       </c>
       <c r="J111" s="29" t="n">
-        <v>0.0011</v>
-      </c>
-      <c r="K111" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1545</v>
+      </c>
+      <c r="K111" s="31" t="n">
+        <v>-0.09300000000000001</v>
       </c>
       <c r="L111" s="28" t="inlineStr">
         <is>
-          <t>0.10~0.29%</t>
+          <t>0.34~0.89%</t>
         </is>
       </c>
       <c r="M111" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.3% · 변동성 0.1% (위험대비 4.09) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.10% · 가장 나쁜 창 연3.0%</t>
+          <t>3해 연21.4% · 변동성 15.4% (위험대비 1.20) (달 간격) · 최대낙폭 -9% · 보수 0.34% · 가장 나쁜 창 연21.4%</t>
         </is>
       </c>
     </row>
@@ -8988,22 +8970,22 @@
       </c>
       <c r="C112" s="33" t="inlineStr">
         <is>
-          <t>NH-Amundi하나로단기채증권투자신탁[채권]</t>
+          <t>마이다스K200인덱스알파증권자투자신탁(주식-파생형)(운용)</t>
         </is>
       </c>
       <c r="D112" s="33" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E112" s="33" t="inlineStr">
         <is>
-          <t>엔에이치아문디자산운용</t>
+          <t>마이다스에셋자산운용</t>
         </is>
       </c>
       <c r="F112" s="34" t="inlineStr">
         <is>
-          <t>3,586억원</t>
+          <t>493억원</t>
         </is>
       </c>
       <c r="G112" s="35" t="inlineStr">
@@ -9013,28 +8995,26 @@
       </c>
       <c r="H112" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I112" s="36" t="n">
-        <v>0.0369</v>
+        <v>0.509</v>
       </c>
       <c r="J112" s="36" t="n">
-        <v>0.0019</v>
-      </c>
-      <c r="K112" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.3986</v>
+      </c>
+      <c r="K112" s="37" t="n">
+        <v>-0.2336</v>
       </c>
       <c r="L112" s="34" t="inlineStr">
         <is>
-          <t>0.10~0.40%</t>
+          <t>0.06~0.15%</t>
         </is>
       </c>
       <c r="M112" s="38" t="inlineStr">
         <is>
-          <t>5해 연3.7% · 변동성 0.2% (위험대비 4.63) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.10% · 가장 나쁜 창 연3.0%</t>
+          <t>3해 연50.9% · 변동성 39.9% (위험대비 1.21) (달 간격) · 최대낙폭 -23% · 보수 0.06% · 가장 나쁜 창 연50.9%</t>
         </is>
       </c>
     </row>
@@ -9051,22 +9031,22 @@
       </c>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>코레이트더블루B증권투자신탁[채권]운용</t>
+          <t>신한퇴직연금커버드콜인덱스증권자투자신탁[주식혼합-파생형] (종류)</t>
         </is>
       </c>
       <c r="D113" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내혼합형</t>
         </is>
       </c>
       <c r="E113" s="14" t="inlineStr">
         <is>
-          <t>코레이트자산운용</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="F113" s="28" t="inlineStr">
         <is>
-          <t>168억원</t>
+          <t>150억원</t>
         </is>
       </c>
       <c r="G113" s="30" t="inlineStr">
@@ -9076,26 +9056,26 @@
       </c>
       <c r="H113" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I113" s="29" t="n">
-        <v>0.0421</v>
+        <v>0.1302</v>
       </c>
       <c r="J113" s="29" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="K113" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L113" s="39" t="n">
-        <v>0.0013</v>
+        <v>0.0872</v>
+      </c>
+      <c r="K113" s="31" t="n">
+        <v>-0.055</v>
+      </c>
+      <c r="L113" s="28" t="inlineStr">
+        <is>
+          <t>0.56~0.79%</t>
+        </is>
       </c>
       <c r="M113" s="32" t="inlineStr">
         <is>
-          <t>5해 연4.2% · 변동성 0.1% (위험대비 14.00) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.13% · 가장 나쁜 창 연3.8%</t>
+          <t>3해 연13.0% · 변동성 8.7% (위험대비 1.17) (달 간격) · 최대낙폭 -6% · 보수 0.56% · 가장 나쁜 창 연13.0%</t>
         </is>
       </c>
     </row>
@@ -9112,22 +9092,22 @@
       </c>
       <c r="C114" s="33" t="inlineStr">
         <is>
-          <t>하나파워e단기채증권자투자신탁[채권]</t>
+          <t>신영밸류고배당증권자투자신탁(주식)운용</t>
         </is>
       </c>
       <c r="D114" s="33" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E114" s="33" t="inlineStr">
         <is>
-          <t>하나자산운용</t>
+          <t>신영자산운용</t>
         </is>
       </c>
       <c r="F114" s="34" t="inlineStr">
         <is>
-          <t>4,958억원</t>
+          <t>8,313억원</t>
         </is>
       </c>
       <c r="G114" s="35" t="inlineStr">
@@ -9137,28 +9117,26 @@
       </c>
       <c r="H114" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I114" s="36" t="n">
-        <v>0.0361</v>
+        <v>0.3287</v>
       </c>
       <c r="J114" s="36" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K114" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.2543</v>
+      </c>
+      <c r="K114" s="37" t="n">
+        <v>-0.1498</v>
       </c>
       <c r="L114" s="34" t="inlineStr">
         <is>
-          <t>0.07~0.19%</t>
+          <t>0.45~1.35%</t>
         </is>
       </c>
       <c r="M114" s="38" t="inlineStr">
         <is>
-          <t>5해 연3.6% · 변동성 0.3% (위험대비 2.86) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.07% · 가장 나쁜 창 연2.9%</t>
+          <t>3해 연32.9% · 변동성 25.4% (위험대비 1.18) (달 간격) · 최대낙폭 -15% · 보수 0.45% · 가장 나쁜 창 연32.9%</t>
         </is>
       </c>
     </row>
@@ -9175,22 +9153,22 @@
       </c>
       <c r="C115" s="14" t="inlineStr">
         <is>
-          <t>베어링고배당플러스증권투자신탁(주식)</t>
+          <t>신한커버드콜인덱스증권자투자신탁[주식혼합-파생형]</t>
         </is>
       </c>
       <c r="D115" s="14" t="inlineStr">
         <is>
-          <t>국내주식형</t>
+          <t>국내혼합형</t>
         </is>
       </c>
       <c r="E115" s="14" t="inlineStr">
         <is>
-          <t>베어링자산운용</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="F115" s="28" t="inlineStr">
         <is>
-          <t>1,834억원</t>
+          <t>161억원</t>
         </is>
       </c>
       <c r="G115" s="30" t="inlineStr">
@@ -9204,24 +9182,22 @@
         </is>
       </c>
       <c r="I115" s="29" t="n">
-        <v>0.3617</v>
+        <v>0.223</v>
       </c>
       <c r="J115" s="29" t="n">
-        <v>0.277</v>
-      </c>
-      <c r="K115" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1433</v>
+      </c>
+      <c r="K115" s="31" t="n">
+        <v>-0.1049</v>
       </c>
       <c r="L115" s="28" t="inlineStr">
         <is>
-          <t>0.33~0.33%</t>
+          <t>0.54~1.34%</t>
         </is>
       </c>
       <c r="M115" s="32" t="inlineStr">
         <is>
-          <t>3해 연36.2% · 변동성 27.7% (위험대비 1.20) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.33% · 가장 나쁜 창 연36.2%</t>
+          <t>3해 연22.3% · 변동성 14.3% (위험대비 1.36) (달 간격) · 최대낙폭 -10% · 보수 0.54% · 가장 나쁜 창 연22.3%</t>
         </is>
       </c>
     </row>
@@ -9238,22 +9214,22 @@
       </c>
       <c r="C116" s="33" t="inlineStr">
         <is>
-          <t>현대머니마켓플렉스증권자투자신탁 1[채권](운용)</t>
+          <t>대신KOSPI200인덱스증권자투자신탁[주식](운용)</t>
         </is>
       </c>
       <c r="D116" s="33" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E116" s="33" t="inlineStr">
         <is>
-          <t>현대자산운용</t>
+          <t>대신자산운용</t>
         </is>
       </c>
       <c r="F116" s="34" t="inlineStr">
         <is>
-          <t>188억원</t>
+          <t>580억원</t>
         </is>
       </c>
       <c r="G116" s="35" t="inlineStr">
@@ -9263,28 +9239,26 @@
       </c>
       <c r="H116" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I116" s="36" t="n">
-        <v>0.0352</v>
+        <v>0.4877</v>
       </c>
       <c r="J116" s="36" t="n">
-        <v>0.0018</v>
-      </c>
-      <c r="K116" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.4041</v>
+      </c>
+      <c r="K116" s="37" t="n">
+        <v>-0.237</v>
       </c>
       <c r="L116" s="34" t="inlineStr">
         <is>
-          <t>0.10~0.40%</t>
+          <t>0.20~0.80%</t>
         </is>
       </c>
       <c r="M116" s="38" t="inlineStr">
         <is>
-          <t>5해 연3.5% · 변동성 0.2% (위험대비 3.94) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.10% · 가장 나쁜 창 연2.7%</t>
+          <t>3해 연48.8% · 변동성 40.4% (위험대비 1.14) (달 간격) · 최대낙폭 -24% · 보수 0.20% · 가장 나쁜 창 연48.8%</t>
         </is>
       </c>
     </row>
@@ -9301,22 +9275,22 @@
       </c>
       <c r="C117" s="14" t="inlineStr">
         <is>
-          <t>키움더드림단기채증권투자신탁[채권]</t>
+          <t>BNKK200인덱스증권투자신탁(주식-파생형)</t>
         </is>
       </c>
       <c r="D117" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E117" s="14" t="inlineStr">
         <is>
-          <t>키움투자자산운용</t>
+          <t>비엔케이자산운용</t>
         </is>
       </c>
       <c r="F117" s="28" t="inlineStr">
         <is>
-          <t>1조원</t>
+          <t>515억원</t>
         </is>
       </c>
       <c r="G117" s="30" t="inlineStr">
@@ -9326,28 +9300,26 @@
       </c>
       <c r="H117" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I117" s="29" t="n">
-        <v>0.0373</v>
+        <v>0.4905</v>
       </c>
       <c r="J117" s="29" t="n">
-        <v>0.0033</v>
-      </c>
-      <c r="K117" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.408</v>
+      </c>
+      <c r="K117" s="31" t="n">
+        <v>-0.2376</v>
       </c>
       <c r="L117" s="28" t="inlineStr">
         <is>
-          <t>0.07~0.33%</t>
+          <t>0.17~0.95%</t>
         </is>
       </c>
       <c r="M117" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.7% · 변동성 0.3% (위험대비 2.79) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.07% · 가장 나쁜 창 연2.7%</t>
+          <t>3해 연49.0% · 변동성 40.8% (위험대비 1.13) (달 간격) · 최대낙폭 -24% · 보수 0.17% · 가장 나쁜 창 연49.0%</t>
         </is>
       </c>
     </row>
@@ -9364,22 +9336,22 @@
       </c>
       <c r="C118" s="33" t="inlineStr">
         <is>
-          <t>유경공모부동산투자신탁3(운용)</t>
+          <t>미래에셋퇴직플랜KRX100인덱스증권자투자신탁 1(주식혼합)</t>
         </is>
       </c>
       <c r="D118" s="33" t="inlineStr">
         <is>
-          <t>국내대체</t>
+          <t>국내혼합형</t>
         </is>
       </c>
       <c r="E118" s="33" t="inlineStr">
         <is>
-          <t>유경피에스지자산운용</t>
+          <t>미래에셋자산운용</t>
         </is>
       </c>
       <c r="F118" s="34" t="inlineStr">
         <is>
-          <t>1,021억원</t>
+          <t>186억원</t>
         </is>
       </c>
       <c r="G118" s="35" t="inlineStr">
@@ -9389,28 +9361,26 @@
       </c>
       <c r="H118" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I118" s="36" t="n">
-        <v>0.0369</v>
+        <v>0.2895</v>
       </c>
       <c r="J118" s="36" t="n">
-        <v>0.0037</v>
-      </c>
-      <c r="K118" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.2318</v>
+      </c>
+      <c r="K118" s="37" t="n">
+        <v>-0.1349</v>
       </c>
       <c r="L118" s="34" t="inlineStr">
         <is>
-          <t>0.27~0.46%</t>
+          <t>0.44~0.65%</t>
         </is>
       </c>
       <c r="M118" s="38" t="inlineStr">
         <is>
-          <t>5해 연3.7% · 변동성 0.4% (위험대비 2.38) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.27% · 가장 나쁜 창 연0.9%</t>
+          <t>3해 연28.9% · 변동성 23.2% (위험대비 1.13) (달 간격) · 최대낙폭 -13% · 보수 0.44% · 가장 나쁜 창 연28.9%</t>
         </is>
       </c>
     </row>
@@ -9427,7 +9397,7 @@
       </c>
       <c r="C119" s="14" t="inlineStr">
         <is>
-          <t>마이다스K200인덱스알파증권자투자신탁(주식-파생형)(운용)</t>
+          <t>신영마라톤지주회사증권자투자신탁(주식)운용</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
@@ -9437,12 +9407,12 @@
       </c>
       <c r="E119" s="14" t="inlineStr">
         <is>
-          <t>마이다스에셋자산운용</t>
+          <t>신영자산운용</t>
         </is>
       </c>
       <c r="F119" s="28" t="inlineStr">
         <is>
-          <t>493억원</t>
+          <t>316억원</t>
         </is>
       </c>
       <c r="G119" s="30" t="inlineStr">
@@ -9456,24 +9426,22 @@
         </is>
       </c>
       <c r="I119" s="29" t="n">
-        <v>0.5527000000000001</v>
+        <v>0.4483</v>
       </c>
       <c r="J119" s="29" t="n">
-        <v>0.4133</v>
-      </c>
-      <c r="K119" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.3544</v>
+      </c>
+      <c r="K119" s="31" t="n">
+        <v>-0.2314</v>
       </c>
       <c r="L119" s="28" t="inlineStr">
         <is>
-          <t>0.06~0.15%</t>
+          <t>0.52~1.49%</t>
         </is>
       </c>
       <c r="M119" s="32" t="inlineStr">
         <is>
-          <t>3해 연55.3% · 변동성 41.3% (위험대비 1.27) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.06% · 가장 나쁜 창 연55.3%</t>
+          <t>3해 연44.8% · 변동성 35.4% (위험대비 1.19) (달 간격) · 최대낙폭 -23% · 보수 0.52% · 가장 나쁜 창 연44.8%</t>
         </is>
       </c>
     </row>
@@ -9490,22 +9458,22 @@
       </c>
       <c r="C120" s="33" t="inlineStr">
         <is>
-          <t>신한코리아인덱스증권투자신탁[주식-파생형](종류)</t>
+          <t>KB퇴직연금배당40증권자투자신탁(채권혼합)</t>
         </is>
       </c>
       <c r="D120" s="33" t="inlineStr">
         <is>
-          <t>국내주식형</t>
+          <t>국내혼합형</t>
         </is>
       </c>
       <c r="E120" s="33" t="inlineStr">
         <is>
-          <t>신한자산운용</t>
+          <t>케이비자산운용</t>
         </is>
       </c>
       <c r="F120" s="34" t="inlineStr">
         <is>
-          <t>3,697억원</t>
+          <t>1조원</t>
         </is>
       </c>
       <c r="G120" s="35" t="inlineStr">
@@ -9519,24 +9487,22 @@
         </is>
       </c>
       <c r="I120" s="36" t="n">
-        <v>0.5354</v>
+        <v>0.1845</v>
       </c>
       <c r="J120" s="36" t="n">
-        <v>0.4193</v>
-      </c>
-      <c r="K120" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1429</v>
+      </c>
+      <c r="K120" s="37" t="n">
+        <v>-0.0965</v>
       </c>
       <c r="L120" s="34" t="inlineStr">
         <is>
-          <t>0.08~0.10%</t>
+          <t>0.46~0.80%</t>
         </is>
       </c>
       <c r="M120" s="38" t="inlineStr">
         <is>
-          <t>3해 연53.5% · 변동성 41.9% (위험대비 1.21) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.08% · 가장 나쁜 창 연53.5%</t>
+          <t>3해 연18.4% · 변동성 14.3% (위험대비 1.09) (달 간격) · 최대낙폭 -10% · 보수 0.46% · 가장 나쁜 창 연18.4%</t>
         </is>
       </c>
     </row>
@@ -9553,22 +9519,22 @@
       </c>
       <c r="C121" s="14" t="inlineStr">
         <is>
-          <t>유리빠른환매미국성장주증권투자신탁[주식-재간접형]운용</t>
+          <t>KB퇴직연금배당증권자투자신탁(주식)(운용)</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>해외주식형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E121" s="14" t="inlineStr">
         <is>
-          <t>유리자산운용</t>
+          <t>케이비자산운용</t>
         </is>
       </c>
       <c r="F121" s="28" t="inlineStr">
         <is>
-          <t>547억원</t>
+          <t>1,688억원</t>
         </is>
       </c>
       <c r="G121" s="30" t="inlineStr">
@@ -9582,24 +9548,22 @@
         </is>
       </c>
       <c r="I121" s="29" t="n">
-        <v>0.2627</v>
+        <v>0.522</v>
       </c>
       <c r="J121" s="29" t="n">
-        <v>0.214</v>
-      </c>
-      <c r="K121" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.3632</v>
+      </c>
+      <c r="K121" s="31" t="n">
+        <v>-0.2298</v>
       </c>
       <c r="L121" s="28" t="inlineStr">
         <is>
-          <t>0.39~1.34%</t>
+          <t>0.71~1.20%</t>
         </is>
       </c>
       <c r="M121" s="32" t="inlineStr">
         <is>
-          <t>3해 연26.3% · 변동성 21.4% (위험대비 1.10) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.39% · 가장 나쁜 창 연26.3%</t>
+          <t>3해 연52.2% · 변동성 36.3% (위험대비 1.36) (달 간격) · 최대낙폭 -23% · 보수 0.71% · 가장 나쁜 창 연52.2%</t>
         </is>
       </c>
     </row>
@@ -9616,7 +9580,7 @@
       </c>
       <c r="C122" s="33" t="inlineStr">
         <is>
-          <t>iM에셋ALL바른ESG단기채증권투자신탁(채권)</t>
+          <t>BNK내일환매초단기채증권자투자신탁(채권)</t>
         </is>
       </c>
       <c r="D122" s="33" t="inlineStr">
@@ -9626,12 +9590,12 @@
       </c>
       <c r="E122" s="33" t="inlineStr">
         <is>
-          <t>아이엠에셋자산운용</t>
+          <t>비엔케이자산운용</t>
         </is>
       </c>
       <c r="F122" s="34" t="inlineStr">
         <is>
-          <t>266억원</t>
+          <t>182억원</t>
         </is>
       </c>
       <c r="G122" s="35" t="inlineStr">
@@ -9645,24 +9609,22 @@
         </is>
       </c>
       <c r="I122" s="36" t="n">
-        <v>0.0377</v>
+        <v>0.0027</v>
       </c>
       <c r="J122" s="36" t="n">
-        <v>0.0026</v>
-      </c>
-      <c r="K122" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0333</v>
+      </c>
+      <c r="K122" s="37" t="n">
+        <v>-0.03759999999999999</v>
       </c>
       <c r="L122" s="34" t="inlineStr">
         <is>
-          <t>0.12~0.41%</t>
+          <t>0.10~0.29%</t>
         </is>
       </c>
       <c r="M122" s="38" t="inlineStr">
         <is>
-          <t>3해 연3.8% · 변동성 0.3% (위험대비 3.69) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.12% · 가장 나쁜 창 연2.8%</t>
+          <t>3해 연0.3% · 변동성 3.3% (위험대비 -0.76) (달 간격) · 최대낙폭 -4% · 보수 0.10% · 가장 나쁜 창 연0.3%</t>
         </is>
       </c>
     </row>
@@ -9679,22 +9641,22 @@
       </c>
       <c r="C123" s="14" t="inlineStr">
         <is>
-          <t>흥국내일드림초단기채증권투자신탁[채권]</t>
+          <t>미래에셋소득공제장기배당커버드콜액티브증권전환형자투자신탁 1(주식혼합)</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내혼합형</t>
         </is>
       </c>
       <c r="E123" s="14" t="inlineStr">
         <is>
-          <t>흥국자산운용</t>
+          <t>미래에셋자산운용</t>
         </is>
       </c>
       <c r="F123" s="28" t="inlineStr">
         <is>
-          <t>512억원</t>
+          <t>259억원</t>
         </is>
       </c>
       <c r="G123" s="30" t="inlineStr">
@@ -9708,22 +9670,22 @@
         </is>
       </c>
       <c r="I123" s="29" t="n">
-        <v>0.0358</v>
+        <v>0.3794</v>
       </c>
       <c r="J123" s="29" t="n">
-        <v>0.0016</v>
-      </c>
-      <c r="K123" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L123" s="39" t="n">
-        <v>0.0015</v>
+        <v>0.2821</v>
+      </c>
+      <c r="K123" s="31" t="n">
+        <v>-0.2063</v>
+      </c>
+      <c r="L123" s="28" t="inlineStr">
+        <is>
+          <t>0.56~1.04%</t>
+        </is>
       </c>
       <c r="M123" s="32" t="inlineStr">
         <is>
-          <t>3해 연3.6% · 변동성 0.2% (위험대비 4.81) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.15% · 가장 나쁜 창 연2.9%</t>
+          <t>3해 연37.9% · 변동성 28.2% (위험대비 1.25) (달 간격) · 최대낙폭 -21% · 보수 0.56% · 가장 나쁜 창 연37.9%</t>
         </is>
       </c>
     </row>
@@ -9740,7 +9702,7 @@
       </c>
       <c r="C124" s="33" t="inlineStr">
         <is>
-          <t>DB해오름인덱스알파증권투자회사[주식-파생형]운용</t>
+          <t>키움코리아인덱스증권자투자신탁 1[주식]</t>
         </is>
       </c>
       <c r="D124" s="33" t="inlineStr">
@@ -9750,12 +9712,12 @@
       </c>
       <c r="E124" s="33" t="inlineStr">
         <is>
-          <t>디비자산운용</t>
+          <t>키움투자자산운용</t>
         </is>
       </c>
       <c r="F124" s="34" t="inlineStr">
         <is>
-          <t>408억원</t>
+          <t>131억원</t>
         </is>
       </c>
       <c r="G124" s="35" t="inlineStr">
@@ -9769,24 +9731,22 @@
         </is>
       </c>
       <c r="I124" s="36" t="n">
-        <v>0.5334</v>
+        <v>0.4842</v>
       </c>
       <c r="J124" s="36" t="n">
-        <v>0.4216</v>
-      </c>
-      <c r="K124" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.4086</v>
+      </c>
+      <c r="K124" s="37" t="n">
+        <v>-0.2355</v>
       </c>
       <c r="L124" s="34" t="inlineStr">
         <is>
-          <t>0.15~0.84%</t>
+          <t>0.21~1.22%</t>
         </is>
       </c>
       <c r="M124" s="38" t="inlineStr">
         <is>
-          <t>3해 연53.3% · 변동성 42.2% (위험대비 1.20) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.15% · 가장 나쁜 창 연53.3%</t>
+          <t>3해 연48.4% · 변동성 40.9% (위험대비 1.12) (달 간격) · 최대낙폭 -24% · 보수 0.21% · 가장 나쁜 창 연48.4%</t>
         </is>
       </c>
     </row>
@@ -9803,22 +9763,22 @@
       </c>
       <c r="C125" s="14" t="inlineStr">
         <is>
-          <t>KB스타단기채증권자투자신탁(채권)(운용)</t>
+          <t>DB진주찾기증권자투자신탁 1[주식]_운용</t>
         </is>
       </c>
       <c r="D125" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E125" s="14" t="inlineStr">
         <is>
-          <t>케이비자산운용</t>
+          <t>디비자산운용</t>
         </is>
       </c>
       <c r="F125" s="28" t="inlineStr">
         <is>
-          <t>662억원</t>
+          <t>226억원</t>
         </is>
       </c>
       <c r="G125" s="30" t="inlineStr">
@@ -9828,28 +9788,26 @@
       </c>
       <c r="H125" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I125" s="29" t="n">
-        <v>0.0338</v>
+        <v>0.4693</v>
       </c>
       <c r="J125" s="29" t="n">
-        <v>0.0022</v>
-      </c>
-      <c r="K125" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.3312</v>
+      </c>
+      <c r="K125" s="31" t="n">
+        <v>-0.1702</v>
       </c>
       <c r="L125" s="28" t="inlineStr">
         <is>
-          <t>0.11~0.28%</t>
+          <t>0.82~1.78%</t>
         </is>
       </c>
       <c r="M125" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.4% · 변동성 0.2% (위험대비 2.59) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.11% · 가장 나쁜 창 연2.8%</t>
+          <t>3해 연46.9% · 변동성 33.1% (위험대비 1.33) (달 간격) · 최대낙폭 -17% · 보수 0.82% · 가장 나쁜 창 연46.9%</t>
         </is>
       </c>
     </row>
@@ -9866,7 +9824,7 @@
       </c>
       <c r="C126" s="33" t="inlineStr">
         <is>
-          <t>한국투자퇴직연금한국의힘증권자투자신탁 1(주식)</t>
+          <t>교보악사파워인덱스증권자투자신탁 2(주식)(운용)</t>
         </is>
       </c>
       <c r="D126" s="33" t="inlineStr">
@@ -9876,12 +9834,12 @@
       </c>
       <c r="E126" s="33" t="inlineStr">
         <is>
-          <t>한국투자신탁운용</t>
+          <t>교보악사자산운용</t>
         </is>
       </c>
       <c r="F126" s="34" t="inlineStr">
         <is>
-          <t>990억원</t>
+          <t>191억원</t>
         </is>
       </c>
       <c r="G126" s="35" t="inlineStr">
@@ -9895,24 +9853,22 @@
         </is>
       </c>
       <c r="I126" s="36" t="n">
-        <v>0.4576</v>
+        <v>0.4859000000000001</v>
       </c>
       <c r="J126" s="36" t="n">
-        <v>0.3896</v>
-      </c>
-      <c r="K126" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.4063000000000001</v>
+      </c>
+      <c r="K126" s="37" t="n">
+        <v>-0.2397</v>
       </c>
       <c r="L126" s="34" t="inlineStr">
         <is>
-          <t>0.39~1.20%</t>
+          <t>0.28~1.17%</t>
         </is>
       </c>
       <c r="M126" s="38" t="inlineStr">
         <is>
-          <t>3해 연45.8% · 변동성 39.0% (위험대비 1.10) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.39% · 가장 나쁜 창 연45.8%</t>
+          <t>3해 연48.6% · 변동성 40.6% (위험대비 1.13) (달 간격) · 최대낙폭 -24% · 보수 0.28% · 가장 나쁜 창 연48.6%</t>
         </is>
       </c>
     </row>
@@ -9929,22 +9885,22 @@
       </c>
       <c r="C127" s="14" t="inlineStr">
         <is>
-          <t>IBK단기채증권자투자신탁[채권]</t>
+          <t>iM에셋인덱스플러스증권자투자신탁 1(주식-파생형)</t>
         </is>
       </c>
       <c r="D127" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E127" s="14" t="inlineStr">
         <is>
-          <t>아이비케이자산운용</t>
+          <t>아이엠에셋자산운용</t>
         </is>
       </c>
       <c r="F127" s="28" t="inlineStr">
         <is>
-          <t>1,196억원</t>
+          <t>136억원</t>
         </is>
       </c>
       <c r="G127" s="30" t="inlineStr">
@@ -9954,28 +9910,26 @@
       </c>
       <c r="H127" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I127" s="29" t="n">
-        <v>0.0356</v>
+        <v>0.481</v>
       </c>
       <c r="J127" s="29" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="K127" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.4089</v>
+      </c>
+      <c r="K127" s="31" t="n">
+        <v>-0.2383</v>
       </c>
       <c r="L127" s="28" t="inlineStr">
         <is>
-          <t>0.09~0.23%</t>
+          <t>0.04~0.52%</t>
         </is>
       </c>
       <c r="M127" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.6% · 변동성 0.3% (위험대비 2.21) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.09% · 가장 나쁜 창 연2.6%</t>
+          <t>3해 연48.1% · 변동성 40.9% (위험대비 1.11) (달 간격) · 최대낙폭 -24% · 보수 0.04% · 가장 나쁜 창 연48.1%</t>
         </is>
       </c>
     </row>
@@ -9992,22 +9946,22 @@
       </c>
       <c r="C128" s="33" t="inlineStr">
         <is>
-          <t>웰컴베스트단기채증권투자신탁[채권형]</t>
+          <t>카디안코리아인덱스증권자투자신탁[주식]</t>
         </is>
       </c>
       <c r="D128" s="33" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E128" s="33" t="inlineStr">
         <is>
-          <t>웰컴자산운용</t>
+          <t>카디안자산운용</t>
         </is>
       </c>
       <c r="F128" s="34" t="inlineStr">
         <is>
-          <t>389억원</t>
+          <t>235억원</t>
         </is>
       </c>
       <c r="G128" s="35" t="inlineStr">
@@ -10021,24 +9975,22 @@
         </is>
       </c>
       <c r="I128" s="36" t="n">
-        <v>0.0348</v>
+        <v>0.4739</v>
       </c>
       <c r="J128" s="36" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="K128" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.4068</v>
+      </c>
+      <c r="K128" s="37" t="n">
+        <v>-0.2358</v>
       </c>
       <c r="L128" s="34" t="inlineStr">
         <is>
-          <t>0.13~0.29%</t>
+          <t>0.27~0.61%</t>
         </is>
       </c>
       <c r="M128" s="38" t="inlineStr">
         <is>
-          <t>3해 연3.5% · 변동성 0.2% (위험대비 3.19) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.13% · 가장 나쁜 창 연2.9%</t>
+          <t>3해 연47.4% · 변동성 40.7% (위험대비 1.10) (달 간격) · 최대낙폭 -24% · 보수 0.27% · 가장 나쁜 창 연47.4%</t>
         </is>
       </c>
     </row>
@@ -10055,22 +10007,22 @@
       </c>
       <c r="C129" s="14" t="inlineStr">
         <is>
-          <t>우리단기채권증권투자신탁(채권)</t>
+          <t>교보악사파워인덱스증권자투자신탁 1(주식)(운용)</t>
         </is>
       </c>
       <c r="D129" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E129" s="14" t="inlineStr">
         <is>
-          <t>우리자산운용</t>
+          <t>교보악사자산운용</t>
         </is>
       </c>
       <c r="F129" s="28" t="inlineStr">
         <is>
-          <t>8,118억원</t>
+          <t>2,914억원</t>
         </is>
       </c>
       <c r="G129" s="30" t="inlineStr">
@@ -10080,28 +10032,26 @@
       </c>
       <c r="H129" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I129" s="29" t="n">
-        <v>0.0372</v>
+        <v>0.4796</v>
       </c>
       <c r="J129" s="29" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="K129" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.4089</v>
+      </c>
+      <c r="K129" s="31" t="n">
+        <v>-0.2396</v>
       </c>
       <c r="L129" s="28" t="inlineStr">
         <is>
-          <t>0.10~0.45%</t>
+          <t>0.17~1.28%</t>
         </is>
       </c>
       <c r="M129" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.7% · 변동성 0.4% (위험대비 2.33) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.10% · 가장 나쁜 창 연2.7%</t>
+          <t>3해 연48.0% · 변동성 40.9% (위험대비 1.10) (달 간격) · 최대낙폭 -24% · 보수 0.17% · 가장 나쁜 창 연48.0%</t>
         </is>
       </c>
     </row>
@@ -10118,22 +10068,22 @@
       </c>
       <c r="C130" s="33" t="inlineStr">
         <is>
-          <t>한화내일받는단기국공채증권자투자신탁(채권)</t>
+          <t>다올퇴직연금40증권자투자신탁[채권혼합](운)</t>
         </is>
       </c>
       <c r="D130" s="33" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내혼합형</t>
         </is>
       </c>
       <c r="E130" s="33" t="inlineStr">
         <is>
-          <t>한화자산운용</t>
+          <t>다올자산운용</t>
         </is>
       </c>
       <c r="F130" s="34" t="inlineStr">
         <is>
-          <t>3,825억원</t>
+          <t>193억원</t>
         </is>
       </c>
       <c r="G130" s="35" t="inlineStr">
@@ -10143,28 +10093,26 @@
       </c>
       <c r="H130" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I130" s="36" t="n">
-        <v>0.0317</v>
+        <v>0.1779</v>
       </c>
       <c r="J130" s="36" t="n">
-        <v>0.0022</v>
-      </c>
-      <c r="K130" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1425</v>
+      </c>
+      <c r="K130" s="37" t="n">
+        <v>-0.0872</v>
       </c>
       <c r="L130" s="34" t="inlineStr">
         <is>
-          <t>0.10~0.25%</t>
+          <t>0.53~0.80%</t>
         </is>
       </c>
       <c r="M130" s="38" t="inlineStr">
         <is>
-          <t>5해 연3.2% · 변동성 0.2% (위험대비 1.64) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.10% · 가장 나쁜 창 연2.7%</t>
+          <t>3해 연17.8% · 변동성 14.2% (위험대비 1.05) (달 간격) · 최대낙폭 -9% · 보수 0.53% · 가장 나쁜 창 연17.8%</t>
         </is>
       </c>
     </row>
@@ -10181,22 +10129,22 @@
       </c>
       <c r="C131" s="14" t="inlineStr">
         <is>
-          <t>현대인베스트먼트단기증권자투자신탁 1(채권)</t>
+          <t>트러스톤인덱스알파증권자투자신탁[주식-파생형]</t>
         </is>
       </c>
       <c r="D131" s="14" t="inlineStr">
         <is>
-          <t>국내채권형</t>
+          <t>국내주식형</t>
         </is>
       </c>
       <c r="E131" s="14" t="inlineStr">
         <is>
-          <t>현대인베스트먼트자산운용</t>
+          <t>트러스톤자산운용</t>
         </is>
       </c>
       <c r="F131" s="28" t="inlineStr">
         <is>
-          <t>915억원</t>
+          <t>326억원</t>
         </is>
       </c>
       <c r="G131" s="30" t="inlineStr">
@@ -10206,28 +10154,26 @@
       </c>
       <c r="H131" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I131" s="29" t="n">
-        <v>0.0315</v>
+        <v>0.478</v>
       </c>
       <c r="J131" s="29" t="n">
-        <v>0.0023</v>
-      </c>
-      <c r="K131" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.4094</v>
+      </c>
+      <c r="K131" s="31" t="n">
+        <v>-0.2398</v>
       </c>
       <c r="L131" s="28" t="inlineStr">
         <is>
-          <t>0.10~0.30%</t>
+          <t>0.10~0.89%</t>
         </is>
       </c>
       <c r="M131" s="32" t="inlineStr">
         <is>
-          <t>5해 연3.1% · 변동성 0.2% (위험대비 1.48) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.10% · 가장 나쁜 창 연2.7%</t>
+          <t>3해 연47.8% · 변동성 40.9% (위험대비 1.10) (달 간격) · 최대낙폭 -24% · 보수 0.10% · 가장 나쁜 창 연47.8%</t>
         </is>
       </c>
     </row>
@@ -10244,22 +10190,22 @@
       </c>
       <c r="C132" s="33" t="inlineStr">
         <is>
-          <t>신한누버거버먼미국가치주증권투자신탁(H)[주식-재간접형](종류)</t>
+          <t>삼성누버거버먼이머징단기채권증권자투자신탁H[채권-재간접형]</t>
         </is>
       </c>
       <c r="D132" s="33" t="inlineStr">
         <is>
-          <t>해외주식형</t>
+          <t>해외채권형</t>
         </is>
       </c>
       <c r="E132" s="33" t="inlineStr">
         <is>
-          <t>신한자산운용</t>
+          <t>삼성자산운용</t>
         </is>
       </c>
       <c r="F132" s="34" t="inlineStr">
         <is>
-          <t>655억원</t>
+          <t>237억원</t>
         </is>
       </c>
       <c r="G132" s="35" t="inlineStr">
@@ -10273,24 +10219,22 @@
         </is>
       </c>
       <c r="I132" s="36" t="n">
-        <v>0.1494</v>
+        <v>0.0607</v>
       </c>
       <c r="J132" s="36" t="n">
-        <v>0.08990000000000001</v>
-      </c>
-      <c r="K132" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0228</v>
+      </c>
+      <c r="K132" s="37" t="n">
+        <v>-0.0179</v>
       </c>
       <c r="L132" s="34" t="inlineStr">
         <is>
-          <t>0.35~1.35%</t>
+          <t>0.23~1.13%</t>
         </is>
       </c>
       <c r="M132" s="38" t="inlineStr">
         <is>
-          <t>3해 연14.9% · 변동성 9.0% (위험대비 1.35) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.35% · 가장 나쁜 창 연14.9%</t>
+          <t>3해 연6.1% · 변동성 2.3% (위험대비 1.43) (달 간격) · 최대낙폭 -2% · 보수 0.23% · 가장 나쁜 창 연3.7%</t>
         </is>
       </c>
     </row>
@@ -10307,7 +10251,7 @@
       </c>
       <c r="C133" s="14" t="inlineStr">
         <is>
-          <t>신한미국S&amp;P500인덱스증권자투자신탁(H)[주식-파생형]</t>
+          <t>미래에셋MSCIAC월드인덱스증권자투자신탁(주식)(UH)</t>
         </is>
       </c>
       <c r="D133" s="14" t="inlineStr">
@@ -10317,12 +10261,12 @@
       </c>
       <c r="E133" s="14" t="inlineStr">
         <is>
-          <t>신한자산운용</t>
+          <t>미래에셋자산운용</t>
         </is>
       </c>
       <c r="F133" s="28" t="inlineStr">
         <is>
-          <t>1,207억원</t>
+          <t>133억원</t>
         </is>
       </c>
       <c r="G133" s="30" t="inlineStr">
@@ -10336,24 +10280,22 @@
         </is>
       </c>
       <c r="I133" s="29" t="n">
-        <v>0.1789</v>
+        <v>0.2023</v>
       </c>
       <c r="J133" s="29" t="n">
-        <v>0.1229</v>
-      </c>
-      <c r="K133" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1124</v>
+      </c>
+      <c r="K133" s="31" t="n">
+        <v>-0.08460000000000001</v>
       </c>
       <c r="L133" s="28" t="inlineStr">
         <is>
-          <t>0.14~1.15%</t>
+          <t>0.27~0.97%</t>
         </is>
       </c>
       <c r="M133" s="32" t="inlineStr">
         <is>
-          <t>3해 연17.9% · 변동성 12.3% (위험대비 1.23) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.14% · 가장 나쁜 창 연15.8%</t>
+          <t>3해 연20.2% · 변동성 11.2% (위험대비 1.55) (달 간격) · 최대낙폭 -8% · 보수 0.27% · 가장 나쁜 창 연19.1%</t>
         </is>
       </c>
     </row>
@@ -10370,7 +10312,7 @@
       </c>
       <c r="C134" s="33" t="inlineStr">
         <is>
-          <t>삼성글로벌배당성장주증권자투자신탁H[주식]</t>
+          <t>피델리티재팬증권자투자신탁(주식-재간접형)</t>
         </is>
       </c>
       <c r="D134" s="33" t="inlineStr">
@@ -10380,12 +10322,12 @@
       </c>
       <c r="E134" s="33" t="inlineStr">
         <is>
-          <t>삼성자산운용</t>
+          <t>피델리티자산운용</t>
         </is>
       </c>
       <c r="F134" s="34" t="inlineStr">
         <is>
-          <t>278억원</t>
+          <t>156억원</t>
         </is>
       </c>
       <c r="G134" s="35" t="inlineStr">
@@ -10399,24 +10341,22 @@
         </is>
       </c>
       <c r="I134" s="36" t="n">
-        <v>0.1427</v>
+        <v>0.2701</v>
       </c>
       <c r="J134" s="36" t="n">
-        <v>0.08800000000000001</v>
-      </c>
-      <c r="K134" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1494</v>
+      </c>
+      <c r="K134" s="37" t="n">
+        <v>-0.0944</v>
       </c>
       <c r="L134" s="34" t="inlineStr">
         <is>
-          <t>0.49~1.49%</t>
+          <t>0.16~1.66%</t>
         </is>
       </c>
       <c r="M134" s="38" t="inlineStr">
         <is>
-          <t>3해 연14.3% · 변동성 8.8% (위험대비 1.30) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.49% · 가장 나쁜 창 연14.3%</t>
+          <t>3해 연27.0% · 변동성 14.9% (위험대비 1.62) (달 간격) · 최대낙폭 -9% · 보수 0.16% · 가장 나쁜 창 연27.0%</t>
         </is>
       </c>
     </row>
@@ -10433,7 +10373,7 @@
       </c>
       <c r="C135" s="14" t="inlineStr">
         <is>
-          <t>삼성글로벌배당성장주증권자투자신탁UH[주식]</t>
+          <t>피델리티글로벌배당인컴증권자투자신탁(주식-재간접형)</t>
         </is>
       </c>
       <c r="D135" s="14" t="inlineStr">
@@ -10443,12 +10383,12 @@
       </c>
       <c r="E135" s="14" t="inlineStr">
         <is>
-          <t>삼성자산운용</t>
+          <t>피델리티자산운용</t>
         </is>
       </c>
       <c r="F135" s="28" t="inlineStr">
         <is>
-          <t>133억원</t>
+          <t>5,716억원</t>
         </is>
       </c>
       <c r="G135" s="30" t="inlineStr">
@@ -10462,24 +10402,22 @@
         </is>
       </c>
       <c r="I135" s="29" t="n">
-        <v>0.1707</v>
+        <v>0.1371</v>
       </c>
       <c r="J135" s="29" t="n">
-        <v>0.1115</v>
-      </c>
-      <c r="K135" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.08130000000000001</v>
+      </c>
+      <c r="K135" s="31" t="n">
+        <v>-0.0654</v>
       </c>
       <c r="L135" s="28" t="inlineStr">
         <is>
-          <t>0.49~1.49%</t>
+          <t>0.16~1.36%</t>
         </is>
       </c>
       <c r="M135" s="32" t="inlineStr">
         <is>
-          <t>3해 연17.1% · 변동성 11.2% (위험대비 1.28) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.49% · 가장 나쁜 창 연17.0%</t>
+          <t>3해 연13.7% · 변동성 8.1% (위험대비 1.34) (달 간격) · 최대낙폭 -7% · 보수 0.16% · 가장 나쁜 창 연13.2%</t>
         </is>
       </c>
     </row>
@@ -10496,22 +10434,22 @@
       </c>
       <c r="C136" s="33" t="inlineStr">
         <is>
-          <t>미래에셋연금동행TRF성장형혼합자산투자신탁(재간접형)</t>
+          <t>KB연금미국S&amp;P500인덱스증권자투자신탁(주식-파생형)(H)(운용)</t>
         </is>
       </c>
       <c r="D136" s="33" t="inlineStr">
         <is>
-          <t>해외혼합형</t>
+          <t>해외주식형</t>
         </is>
       </c>
       <c r="E136" s="33" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>케이비자산운용</t>
         </is>
       </c>
       <c r="F136" s="34" t="inlineStr">
         <is>
-          <t>1,276억원</t>
+          <t>1,626억원</t>
         </is>
       </c>
       <c r="G136" s="35" t="inlineStr">
@@ -10525,24 +10463,22 @@
         </is>
       </c>
       <c r="I136" s="36" t="n">
-        <v>0.1715</v>
+        <v>0.2086</v>
       </c>
       <c r="J136" s="36" t="n">
-        <v>0.1271</v>
-      </c>
-      <c r="K136" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1193</v>
+      </c>
+      <c r="K136" s="37" t="n">
+        <v>-0.08380000000000001</v>
       </c>
       <c r="L136" s="34" t="inlineStr">
         <is>
-          <t>0.55~0.81%</t>
+          <t>0.67~1.23%</t>
         </is>
       </c>
       <c r="M136" s="38" t="inlineStr">
         <is>
-          <t>3해 연17.1% · 변동성 12.7% (위험대비 1.13) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.55% · 가장 나쁜 창 연17.1%</t>
+          <t>3해 연20.9% · 변동성 11.9% (위험대비 1.51) (달 간격) · 최대낙폭 -8% · 보수 0.67% · 가장 나쁜 창 연20.9%</t>
         </is>
       </c>
     </row>
@@ -10559,22 +10495,22 @@
       </c>
       <c r="C137" s="14" t="inlineStr">
         <is>
-          <t>미래에셋글로벌자산배분밸런스형증권투자신탁(혼합-재간접형)(UH)</t>
+          <t>신한누버거버먼미국가치주증권투자신탁(H)[주식-재간접형](종류)</t>
         </is>
       </c>
       <c r="D137" s="14" t="inlineStr">
         <is>
-          <t>해외혼합형</t>
+          <t>해외주식형</t>
         </is>
       </c>
       <c r="E137" s="14" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="F137" s="28" t="inlineStr">
         <is>
-          <t>231억원</t>
+          <t>655억원</t>
         </is>
       </c>
       <c r="G137" s="30" t="inlineStr">
@@ -10588,24 +10524,22 @@
         </is>
       </c>
       <c r="I137" s="29" t="n">
-        <v>0.1788</v>
+        <v>0.1478</v>
       </c>
       <c r="J137" s="29" t="n">
-        <v>0.1303</v>
-      </c>
-      <c r="K137" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1007</v>
+      </c>
+      <c r="K137" s="31" t="n">
+        <v>-0.0694</v>
       </c>
       <c r="L137" s="28" t="inlineStr">
         <is>
-          <t>0.40~1.20%</t>
+          <t>0.35~1.35%</t>
         </is>
       </c>
       <c r="M137" s="32" t="inlineStr">
         <is>
-          <t>3해 연17.9% · 변동성 13.0% (위험대비 1.16) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.40% · 가장 나쁜 창 연14.4%</t>
+          <t>3해 연14.8% · 변동성 10.1% (위험대비 1.19) (달 간격) · 최대낙폭 -7% · 보수 0.35% · 가장 나쁜 창 연14.8%</t>
         </is>
       </c>
     </row>
@@ -10622,7 +10556,7 @@
       </c>
       <c r="C138" s="33" t="inlineStr">
         <is>
-          <t>KB타겟리턴적극형OCIO증권투자신탁(혼합-재간접형)(운용)</t>
+          <t>NH-AmundiSignatureOCIO성장형증권자투자신탁(UH)[혼합-재간접형]</t>
         </is>
       </c>
       <c r="D138" s="33" t="inlineStr">
@@ -10632,12 +10566,12 @@
       </c>
       <c r="E138" s="33" t="inlineStr">
         <is>
-          <t>케이비자산운용</t>
+          <t>엔에이치아문디자산운용</t>
         </is>
       </c>
       <c r="F138" s="34" t="inlineStr">
         <is>
-          <t>234억원</t>
+          <t>155억원</t>
         </is>
       </c>
       <c r="G138" s="35" t="inlineStr">
@@ -10651,24 +10585,22 @@
         </is>
       </c>
       <c r="I138" s="36" t="n">
-        <v>0.1491</v>
+        <v>0.1817</v>
       </c>
       <c r="J138" s="36" t="n">
-        <v>0.1131</v>
-      </c>
-      <c r="K138" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.09859999999999999</v>
+      </c>
+      <c r="K138" s="37" t="n">
+        <v>-0.0814</v>
       </c>
       <c r="L138" s="34" t="inlineStr">
         <is>
-          <t>0.55~0.82%</t>
+          <t>0.79~1.39%</t>
         </is>
       </c>
       <c r="M138" s="38" t="inlineStr">
         <is>
-          <t>3해 연14.9% · 변동성 11.3% (위험대비 1.07) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.55% · 가장 나쁜 창 연14.9%</t>
+          <t>3해 연18.2% · 변동성 9.9% (위험대비 1.56) (달 간격) · 최대낙폭 -8% · 보수 0.79% · 가장 나쁜 창 연16.7%</t>
         </is>
       </c>
     </row>
@@ -10685,22 +10617,22 @@
       </c>
       <c r="C139" s="14" t="inlineStr">
         <is>
-          <t>NH-AmundiSignatureOCIO성장형증권자투자신탁(UH)[혼합-재간접형]</t>
+          <t>AB셀렉트미국증권투자신탁(주식-재간접형)</t>
         </is>
       </c>
       <c r="D139" s="14" t="inlineStr">
         <is>
-          <t>해외혼합형</t>
+          <t>해외주식형</t>
         </is>
       </c>
       <c r="E139" s="14" t="inlineStr">
         <is>
-          <t>엔에이치아문디자산운용</t>
+          <t>얼라이언스번스틴자산운용</t>
         </is>
       </c>
       <c r="F139" s="28" t="inlineStr">
         <is>
-          <t>155억원</t>
+          <t>305억원</t>
         </is>
       </c>
       <c r="G139" s="30" t="inlineStr">
@@ -10714,24 +10646,22 @@
         </is>
       </c>
       <c r="I139" s="29" t="n">
-        <v>0.1797</v>
+        <v>0.1761</v>
       </c>
       <c r="J139" s="29" t="n">
-        <v>0.1123</v>
-      </c>
-      <c r="K139" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1169</v>
+      </c>
+      <c r="K139" s="31" t="n">
+        <v>-0.07870000000000001</v>
       </c>
       <c r="L139" s="28" t="inlineStr">
         <is>
-          <t>0.79~1.39%</t>
+          <t>0.27~1.56%</t>
         </is>
       </c>
       <c r="M139" s="32" t="inlineStr">
         <is>
-          <t>3해 연18.0% · 변동성 11.2% (위험대비 1.35) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.79% · 가장 나쁜 창 연13.7%</t>
+          <t>3해 연17.6% · 변동성 11.7% (위험대비 1.27) (달 간격) · 최대낙폭 -8% · 보수 0.27% · 가장 나쁜 창 연14.5%</t>
         </is>
       </c>
     </row>
@@ -10748,22 +10678,22 @@
       </c>
       <c r="C140" s="33" t="inlineStr">
         <is>
-          <t>NH-AmundiSignatureOCIO성장형증권자투자신탁(H)[혼합-재간접형]</t>
+          <t>AB글로벌고수익증권투자신탁(채권-재간접형)</t>
         </is>
       </c>
       <c r="D140" s="33" t="inlineStr">
         <is>
-          <t>해외혼합형</t>
+          <t>해외채권형</t>
         </is>
       </c>
       <c r="E140" s="33" t="inlineStr">
         <is>
-          <t>엔에이치아문디자산운용</t>
+          <t>얼라이언스번스틴자산운용</t>
         </is>
       </c>
       <c r="F140" s="34" t="inlineStr">
         <is>
-          <t>356억원</t>
+          <t>1,629억원</t>
         </is>
       </c>
       <c r="G140" s="35" t="inlineStr">
@@ -10777,24 +10707,22 @@
         </is>
       </c>
       <c r="I140" s="36" t="n">
-        <v>0.1486</v>
+        <v>0.0614</v>
       </c>
       <c r="J140" s="36" t="n">
-        <v>0.09910000000000001</v>
-      </c>
-      <c r="K140" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.04389999999999999</v>
+      </c>
+      <c r="K140" s="37" t="n">
+        <v>-0.026</v>
       </c>
       <c r="L140" s="34" t="inlineStr">
         <is>
-          <t>0.79~1.39%</t>
+          <t>0.17~1.17%</t>
         </is>
       </c>
       <c r="M140" s="38" t="inlineStr">
         <is>
-          <t>3해 연14.9% · 변동성 9.9% (위험대비 1.22) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.79% · 가장 나쁜 창 연14.3%</t>
+          <t>3해 연6.1% · 변동성 4.4% (위험대비 0.76) (달 간격) · 최대낙폭 -3% · 보수 0.17% · 가장 나쁜 창 연2.9%</t>
         </is>
       </c>
     </row>
@@ -10811,22 +10739,22 @@
       </c>
       <c r="C141" s="14" t="inlineStr">
         <is>
-          <t>iM에셋디딤코어EMP증권투자신탁(혼합-재간접형)</t>
+          <t>미래에셋미국배당커버드콜액티브증권자투자신탁(주식)(H)</t>
         </is>
       </c>
       <c r="D141" s="14" t="inlineStr">
         <is>
-          <t>해외혼합형</t>
+          <t>해외주식형</t>
         </is>
       </c>
       <c r="E141" s="14" t="inlineStr">
         <is>
-          <t>아이엠에셋자산운용</t>
+          <t>미래에셋자산운용</t>
         </is>
       </c>
       <c r="F141" s="28" t="inlineStr">
         <is>
-          <t>217억원</t>
+          <t>234억원</t>
         </is>
       </c>
       <c r="G141" s="30" t="inlineStr">
@@ -10840,24 +10768,22 @@
         </is>
       </c>
       <c r="I141" s="29" t="n">
-        <v>0.1115</v>
+        <v>0.165</v>
       </c>
       <c r="J141" s="29" t="n">
-        <v>0.0873</v>
-      </c>
-      <c r="K141" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1046</v>
+      </c>
+      <c r="K141" s="31" t="n">
+        <v>-0.0725</v>
       </c>
       <c r="L141" s="28" t="inlineStr">
         <is>
-          <t>0.54~1.46%</t>
+          <t>0.66~1.86%</t>
         </is>
       </c>
       <c r="M141" s="32" t="inlineStr">
         <is>
-          <t>3해 연11.2% · 변동성 8.7% (위험대비 0.96) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.54% · 가장 나쁜 창 연11.2%</t>
+          <t>3해 연16.5% · 변동성 10.5% (위험대비 1.31) (달 간격) · 최대낙폭 -7% · 보수 0.66% · 가장 나쁜 창 연16.1%</t>
         </is>
       </c>
     </row>
@@ -10874,7 +10800,7 @@
       </c>
       <c r="C142" s="33" t="inlineStr">
         <is>
-          <t>AB셀렉트미국증권투자신탁(주식-재간접형)</t>
+          <t>신한동유럽플러스증권자투자신탁(H)[주식](종류)</t>
         </is>
       </c>
       <c r="D142" s="33" t="inlineStr">
@@ -10884,12 +10810,12 @@
       </c>
       <c r="E142" s="33" t="inlineStr">
         <is>
-          <t>얼라이언스번스틴자산운용</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="F142" s="34" t="inlineStr">
         <is>
-          <t>305억원</t>
+          <t>139억원</t>
         </is>
       </c>
       <c r="G142" s="35" t="inlineStr">
@@ -10899,28 +10825,26 @@
       </c>
       <c r="H142" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I142" s="36" t="n">
-        <v>0.1012</v>
+        <v>0.2581</v>
       </c>
       <c r="J142" s="36" t="n">
-        <v>0.1016</v>
-      </c>
-      <c r="K142" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1049</v>
+      </c>
+      <c r="K142" s="37" t="n">
+        <v>-0.0503</v>
       </c>
       <c r="L142" s="34" t="inlineStr">
         <is>
-          <t>0.27~1.56%</t>
+          <t>1.11~1.86%</t>
         </is>
       </c>
       <c r="M142" s="38" t="inlineStr">
         <is>
-          <t>5해 연10.1% · 변동성 10.2% (위험대비 0.72) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.27% · 가장 나쁜 창 연10.1%</t>
+          <t>3해 연25.8% · 변동성 10.5% (위험대비 2.19) (달 간격) · 최대낙폭 -5% · 보수 1.11% · 가장 나쁜 창 연23.3%</t>
         </is>
       </c>
     </row>
@@ -10937,22 +10861,22 @@
       </c>
       <c r="C143" s="14" t="inlineStr">
         <is>
-          <t>피델리티재팬증권자투자신탁(주식-재간접형)</t>
+          <t>키움슈로더글로벌타겟리턴증권투자신탁(주식혼합-재간접형)</t>
         </is>
       </c>
       <c r="D143" s="14" t="inlineStr">
         <is>
-          <t>해외주식형</t>
+          <t>해외혼합형</t>
         </is>
       </c>
       <c r="E143" s="14" t="inlineStr">
         <is>
-          <t>피델리티자산운용</t>
+          <t>키움투자자산운용</t>
         </is>
       </c>
       <c r="F143" s="28" t="inlineStr">
         <is>
-          <t>156억원</t>
+          <t>125억원</t>
         </is>
       </c>
       <c r="G143" s="30" t="inlineStr">
@@ -10962,28 +10886,26 @@
       </c>
       <c r="H143" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I143" s="29" t="n">
-        <v>0.2139</v>
+        <v>0.1092</v>
       </c>
       <c r="J143" s="29" t="n">
-        <v>0.2143</v>
-      </c>
-      <c r="K143" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0526</v>
+      </c>
+      <c r="K143" s="31" t="n">
+        <v>-0.0353</v>
       </c>
       <c r="L143" s="28" t="inlineStr">
         <is>
-          <t>0.16~1.66%</t>
+          <t>0.76~1.66%</t>
         </is>
       </c>
       <c r="M143" s="32" t="inlineStr">
         <is>
-          <t>5해 연21.4% · 변동성 21.4% (위험대비 0.87) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.16% · 가장 나쁜 창 연21.4%</t>
+          <t>3해 연10.9% · 변동성 5.3% (위험대비 1.54) (달 간격) · 최대낙폭 -4% · 보수 0.76% · 가장 나쁜 창 연10.9%</t>
         </is>
       </c>
     </row>
@@ -11000,7 +10922,7 @@
       </c>
       <c r="C144" s="33" t="inlineStr">
         <is>
-          <t>한화단기하이일드증권자투자신탁(채권)</t>
+          <t>삼성누버거버먼이머징국공채플러스증권자투자신탁H[채권-재간접형]</t>
         </is>
       </c>
       <c r="D144" s="33" t="inlineStr">
@@ -11010,12 +10932,12 @@
       </c>
       <c r="E144" s="33" t="inlineStr">
         <is>
-          <t>한화자산운용</t>
+          <t>삼성자산운용</t>
         </is>
       </c>
       <c r="F144" s="34" t="inlineStr">
         <is>
-          <t>169억원</t>
+          <t>502억원</t>
         </is>
       </c>
       <c r="G144" s="35" t="inlineStr">
@@ -11025,28 +10947,26 @@
       </c>
       <c r="H144" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I144" s="36" t="n">
-        <v>0.0351</v>
+        <v>0.1075</v>
       </c>
       <c r="J144" s="36" t="n">
-        <v>0.0151</v>
-      </c>
-      <c r="K144" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0621</v>
+      </c>
+      <c r="K144" s="37" t="n">
+        <v>-0.0391</v>
       </c>
       <c r="L144" s="34" t="inlineStr">
         <is>
-          <t>0.71~1.71%</t>
+          <t>0.23~1.13%</t>
         </is>
       </c>
       <c r="M144" s="38" t="inlineStr">
         <is>
-          <t>5해 연3.5% · 변동성 1.5% (위험대비 0.46) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.71% · 가장 나쁜 창 연3.4%</t>
+          <t>3해 연10.8% · 변동성 6.2% (위험대비 1.28) (달 간격) · 최대낙폭 -4% · 보수 0.23% · 가장 나쁜 창 연8.1%</t>
         </is>
       </c>
     </row>
@@ -11063,22 +10983,22 @@
       </c>
       <c r="C145" s="14" t="inlineStr">
         <is>
-          <t>피델리티글로벌배당인컴증권자투자신탁(주식-재간접형)</t>
+          <t>베어링월지급글로벌하이일드증권자투자신탁[H](채권-재간접형)</t>
         </is>
       </c>
       <c r="D145" s="14" t="inlineStr">
         <is>
-          <t>해외주식형</t>
+          <t>해외채권형</t>
         </is>
       </c>
       <c r="E145" s="14" t="inlineStr">
         <is>
-          <t>피델리티자산운용</t>
+          <t>베어링자산운용</t>
         </is>
       </c>
       <c r="F145" s="28" t="inlineStr">
         <is>
-          <t>5,716억원</t>
+          <t>496억원</t>
         </is>
       </c>
       <c r="G145" s="30" t="inlineStr">
@@ -11088,28 +11008,26 @@
       </c>
       <c r="H145" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I145" s="29" t="n">
-        <v>0.08</v>
+        <v>0.06480000000000001</v>
       </c>
       <c r="J145" s="29" t="n">
-        <v>0.08839999999999999</v>
-      </c>
-      <c r="K145" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0339</v>
+      </c>
+      <c r="K145" s="31" t="n">
+        <v>-0.0218</v>
       </c>
       <c r="L145" s="28" t="inlineStr">
         <is>
-          <t>0.16~1.36%</t>
+          <t>0.49~1.19%</t>
         </is>
       </c>
       <c r="M145" s="32" t="inlineStr">
         <is>
-          <t>5해 연8.0% · 변동성 8.8% (위험대비 0.59) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.16% · 가장 나쁜 창 연8.0%</t>
+          <t>3해 연6.5% · 변동성 3.4% (위험대비 1.08) (달 간격) · 최대낙폭 -2% · 보수 0.49% · 가장 나쁜 창 연3.7%</t>
         </is>
       </c>
     </row>
@@ -11126,22 +11044,22 @@
       </c>
       <c r="C146" s="33" t="inlineStr">
         <is>
-          <t>한화연금단기하이일드증권자투자신탁(채권)</t>
+          <t>NH-AmundiSignatureOCIO성장형증권자투자신탁(H)[혼합-재간접형]</t>
         </is>
       </c>
       <c r="D146" s="33" t="inlineStr">
         <is>
-          <t>해외채권형</t>
+          <t>해외혼합형</t>
         </is>
       </c>
       <c r="E146" s="33" t="inlineStr">
         <is>
-          <t>한화자산운용</t>
+          <t>엔에이치아문디자산운용</t>
         </is>
       </c>
       <c r="F146" s="34" t="inlineStr">
         <is>
-          <t>172억원</t>
+          <t>356억원</t>
         </is>
       </c>
       <c r="G146" s="35" t="inlineStr">
@@ -11151,28 +11069,26 @@
       </c>
       <c r="H146" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I146" s="36" t="n">
-        <v>0.035</v>
+        <v>0.1396</v>
       </c>
       <c r="J146" s="36" t="n">
-        <v>0.0156</v>
-      </c>
-      <c r="K146" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0975</v>
+      </c>
+      <c r="K146" s="37" t="n">
+        <v>-0.07240000000000001</v>
       </c>
       <c r="L146" s="34" t="inlineStr">
         <is>
-          <t>0.71~0.97%</t>
+          <t>0.79~1.39%</t>
         </is>
       </c>
       <c r="M146" s="38" t="inlineStr">
         <is>
-          <t>5해 연3.5% · 변동성 1.6% (위험대비 0.44) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.71% · 가장 나쁜 창 연3.4%</t>
+          <t>3해 연14.0% · 변동성 9.8% (위험대비 1.14) (달 간격) · 최대낙폭 -7% · 보수 0.79% · 가장 나쁜 창 연14.0%</t>
         </is>
       </c>
     </row>
@@ -11189,7 +11105,7 @@
       </c>
       <c r="C147" s="14" t="inlineStr">
         <is>
-          <t>iM에셋월드에너지증권자투자신탁(주식-재간접형)(H)</t>
+          <t>한화천연자원증권자투자신탁(주식)</t>
         </is>
       </c>
       <c r="D147" s="14" t="inlineStr">
@@ -11199,12 +11115,12 @@
       </c>
       <c r="E147" s="14" t="inlineStr">
         <is>
-          <t>아이엠에셋자산운용</t>
+          <t>한화자산운용</t>
         </is>
       </c>
       <c r="F147" s="28" t="inlineStr">
         <is>
-          <t>288억원</t>
+          <t>1,120억원</t>
         </is>
       </c>
       <c r="G147" s="30" t="inlineStr">
@@ -11214,28 +11130,26 @@
       </c>
       <c r="H147" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I147" s="29" t="n">
-        <v>0.2359</v>
+        <v>0.2396</v>
       </c>
       <c r="J147" s="29" t="n">
-        <v>0.1806</v>
-      </c>
-      <c r="K147" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1608</v>
+      </c>
+      <c r="K147" s="31" t="n">
+        <v>-0.08460000000000001</v>
       </c>
       <c r="L147" s="28" t="inlineStr">
         <is>
-          <t>0.56~1.66%</t>
+          <t>0.94~2.44%</t>
         </is>
       </c>
       <c r="M147" s="32" t="inlineStr">
         <is>
-          <t>5해 연23.6% · 변동성 18.1% (위험대비 1.15) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.56% · 가장 나쁜 창 연14.4%</t>
+          <t>3해 연24.0% · 변동성 16.1% (위험대비 1.32) (달 간격) · 최대낙폭 -8% · 보수 0.94% · 가장 나쁜 창 연24.0%</t>
         </is>
       </c>
     </row>
@@ -11252,22 +11166,22 @@
       </c>
       <c r="C148" s="33" t="inlineStr">
         <is>
-          <t>한국투자글로벌AI&amp;반도체TOP10증권자투자신탁UH(주식)(모)</t>
+          <t>우리PIMCO분산투자증권자투자신탁[채권_재간접형](H)운용</t>
         </is>
       </c>
       <c r="D148" s="33" t="inlineStr">
         <is>
-          <t>해외주식형</t>
+          <t>해외채권형</t>
         </is>
       </c>
       <c r="E148" s="33" t="inlineStr">
         <is>
-          <t>한국투자신탁운용</t>
+          <t>우리자산운용</t>
         </is>
       </c>
       <c r="F148" s="34" t="inlineStr">
         <is>
-          <t>1,620억원</t>
+          <t>292억원</t>
         </is>
       </c>
       <c r="G148" s="35" t="inlineStr">
@@ -11281,24 +11195,22 @@
         </is>
       </c>
       <c r="I148" s="36" t="n">
-        <v>0.4327</v>
+        <v>0.0582</v>
       </c>
       <c r="J148" s="36" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="K148" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0443</v>
+      </c>
+      <c r="K148" s="37" t="n">
+        <v>-0.0282</v>
       </c>
       <c r="L148" s="34" t="inlineStr">
         <is>
-          <t>0.74~1.74%</t>
+          <t>0.29~1.29%</t>
         </is>
       </c>
       <c r="M148" s="38" t="inlineStr">
         <is>
-          <t>3해 연43.3% · 변동성 29.7% (위험대비 1.36) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.74% · 가장 나쁜 창 연43.3%</t>
+          <t>3해 연5.8% · 변동성 4.4% (위험대비 0.68) (달 간격) · 최대낙폭 -3% · 보수 0.29% · 가장 나쁜 창 연3.1%</t>
         </is>
       </c>
     </row>
@@ -11315,22 +11227,22 @@
       </c>
       <c r="C149" s="14" t="inlineStr">
         <is>
-          <t>KB평생연금밸런스증권자투자신탁(채권혼합-재간접형)(운용)</t>
+          <t>한국투자TIF알아서평생소득증권자투자신탁(채권-재간접형)</t>
         </is>
       </c>
       <c r="D149" s="14" t="inlineStr">
         <is>
-          <t>해외혼합형</t>
+          <t>해외채권형</t>
         </is>
       </c>
       <c r="E149" s="14" t="inlineStr">
         <is>
-          <t>케이비자산운용</t>
+          <t>한국투자신탁운용</t>
         </is>
       </c>
       <c r="F149" s="28" t="inlineStr">
         <is>
-          <t>134억원</t>
+          <t>125억원</t>
         </is>
       </c>
       <c r="G149" s="30" t="inlineStr">
@@ -11344,24 +11256,22 @@
         </is>
       </c>
       <c r="I149" s="29" t="n">
-        <v>0.06059999999999999</v>
+        <v>0.0428</v>
       </c>
       <c r="J149" s="29" t="n">
-        <v>0.05309999999999999</v>
-      </c>
-      <c r="K149" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.0363</v>
+      </c>
+      <c r="K149" s="31" t="n">
+        <v>-0.025</v>
       </c>
       <c r="L149" s="28" t="inlineStr">
         <is>
-          <t>0.30~0.51%</t>
+          <t>0.35~0.82%</t>
         </is>
       </c>
       <c r="M149" s="32" t="inlineStr">
         <is>
-          <t>3해 연6.1% · 변동성 5.3% (위험대비 0.61) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.30% · 가장 나쁜 창 연5.7%</t>
+          <t>3해 연4.3% · 변동성 3.6% (위험대비 0.40) (달 간격) · 최대낙폭 -2% · 보수 0.35% · 가장 나쁜 창 연1.3%</t>
         </is>
       </c>
     </row>
@@ -11378,7 +11288,7 @@
       </c>
       <c r="C150" s="33" t="inlineStr">
         <is>
-          <t>한국투자글로벌AI&amp;반도체TOP10증권자투자신탁H(주식)(모)</t>
+          <t>한국투자웰링턴글로벌퀄리티증권자투자신탁H(주식)</t>
         </is>
       </c>
       <c r="D150" s="33" t="inlineStr">
@@ -11393,7 +11303,7 @@
       </c>
       <c r="F150" s="34" t="inlineStr">
         <is>
-          <t>1,623억원</t>
+          <t>906억원</t>
         </is>
       </c>
       <c r="G150" s="35" t="inlineStr">
@@ -11407,24 +11317,22 @@
         </is>
       </c>
       <c r="I150" s="36" t="n">
-        <v>0.3962</v>
+        <v>0.1715</v>
       </c>
       <c r="J150" s="36" t="n">
-        <v>0.2845</v>
-      </c>
-      <c r="K150" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1123</v>
+      </c>
+      <c r="K150" s="37" t="n">
+        <v>-0.0862</v>
       </c>
       <c r="L150" s="34" t="inlineStr">
         <is>
-          <t>0.74~1.74%</t>
+          <t>0.97~2.17%</t>
         </is>
       </c>
       <c r="M150" s="38" t="inlineStr">
         <is>
-          <t>3해 연39.6% · 변동성 28.4% (위험대비 1.29) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.74% · 가장 나쁜 창 연39.6%</t>
+          <t>3해 연17.1% · 변동성 11.2% (위험대비 1.28) (달 간격) · 최대낙폭 -9% · 보수 0.97% · 가장 나쁜 창 연12.4%</t>
         </is>
       </c>
     </row>
@@ -11441,7 +11349,7 @@
       </c>
       <c r="C151" s="14" t="inlineStr">
         <is>
-          <t>KCGI글로벌고배당증권자투자신탁[주식-재간접형]</t>
+          <t>브이아이아시아넥스트인프라증권자투자신탁 1[주식]</t>
         </is>
       </c>
       <c r="D151" s="14" t="inlineStr">
@@ -11451,12 +11359,12 @@
       </c>
       <c r="E151" s="14" t="inlineStr">
         <is>
-          <t>케이씨지아이자산운용</t>
+          <t>브이아이자산운용</t>
         </is>
       </c>
       <c r="F151" s="28" t="inlineStr">
         <is>
-          <t>189억원</t>
+          <t>127억원</t>
         </is>
       </c>
       <c r="G151" s="30" t="inlineStr">
@@ -11466,28 +11374,26 @@
       </c>
       <c r="H151" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I151" s="29" t="n">
-        <v>0.0902</v>
+        <v>0.1846</v>
       </c>
       <c r="J151" s="29" t="n">
-        <v>0.101</v>
-      </c>
-      <c r="K151" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1316</v>
+      </c>
+      <c r="K151" s="31" t="n">
+        <v>-0.0721</v>
       </c>
       <c r="L151" s="28" t="inlineStr">
         <is>
-          <t>0.49~0.65%</t>
+          <t>1.33~2.08%</t>
         </is>
       </c>
       <c r="M151" s="32" t="inlineStr">
         <is>
-          <t>5해 연9.0% · 변동성 10.1% (위험대비 0.61) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.49% · 가장 나쁜 창 연9.0%</t>
+          <t>3해 연18.5% · 변동성 13.2% (위험대비 1.19) (달 간격) · 최대낙폭 -7% · 보수 1.33% · 가장 나쁜 창 연18.5%</t>
         </is>
       </c>
     </row>
@@ -11504,12 +11410,12 @@
       </c>
       <c r="C152" s="33" t="inlineStr">
         <is>
-          <t>키움불리오글로벌멀티에셋EMP증권자투자신탁(UH)[혼합-재간접형]</t>
+          <t>키움슈로더유로증권자투자신탁(주식-재간접형)</t>
         </is>
       </c>
       <c r="D152" s="33" t="inlineStr">
         <is>
-          <t>해외혼합형</t>
+          <t>해외주식형</t>
         </is>
       </c>
       <c r="E152" s="33" t="inlineStr">
@@ -11519,7 +11425,7 @@
       </c>
       <c r="F152" s="34" t="inlineStr">
         <is>
-          <t>659억원</t>
+          <t>214억원</t>
         </is>
       </c>
       <c r="G152" s="35" t="inlineStr">
@@ -11529,28 +11435,26 @@
       </c>
       <c r="H152" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I152" s="36" t="n">
-        <v>0.1028</v>
+        <v>0.1602</v>
       </c>
       <c r="J152" s="36" t="n">
-        <v>0.1173</v>
-      </c>
-      <c r="K152" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1201</v>
+      </c>
+      <c r="K152" s="37" t="n">
+        <v>-0.0978</v>
       </c>
       <c r="L152" s="34" t="inlineStr">
         <is>
-          <t>0.70~1.57%</t>
+          <t>0.91~2.41%</t>
         </is>
       </c>
       <c r="M152" s="38" t="inlineStr">
         <is>
-          <t>5해 연10.3% · 변동성 11.7% (위험대비 0.64) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.70% · 가장 나쁜 창 연10.3%</t>
+          <t>3해 연16.0% · 변동성 12.0% (위험대비 1.10) (달 간격) · 최대낙폭 -10% · 보수 0.91% · 가장 나쁜 창 연15.1%</t>
         </is>
       </c>
     </row>
@@ -11567,22 +11471,22 @@
       </c>
       <c r="C153" s="14" t="inlineStr">
         <is>
-          <t>키움슈로더월지급글로벌가치주인컴증권자투자신탁[주식-재간접형]</t>
+          <t>하나PIMCO글로벌인컴혼합자산자투자신탁(H)[재간접형]</t>
         </is>
       </c>
       <c r="D153" s="14" t="inlineStr">
         <is>
-          <t>해외주식형</t>
+          <t>해외채권형</t>
         </is>
       </c>
       <c r="E153" s="14" t="inlineStr">
         <is>
-          <t>키움투자자산운용</t>
+          <t>하나자산운용</t>
         </is>
       </c>
       <c r="F153" s="28" t="inlineStr">
         <is>
-          <t>1,713억원</t>
+          <t>700억원</t>
         </is>
       </c>
       <c r="G153" s="30" t="inlineStr">
@@ -11592,28 +11496,26 @@
       </c>
       <c r="H153" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I153" s="29" t="n">
-        <v>0.0755</v>
+        <v>0.0506</v>
       </c>
       <c r="J153" s="29" t="n">
-        <v>0.1013</v>
-      </c>
-      <c r="K153" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.04190000000000001</v>
+      </c>
+      <c r="K153" s="31" t="n">
+        <v>-0.0271</v>
       </c>
       <c r="L153" s="28" t="inlineStr">
         <is>
-          <t>0.43~1.21%</t>
+          <t>0.36~1.16%</t>
         </is>
       </c>
       <c r="M153" s="32" t="inlineStr">
         <is>
-          <t>5해 연7.5% · 변동성 10.1% (위험대비 0.47) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.43% · 가장 나쁜 창 연7.5%</t>
+          <t>3해 연5.1% · 변동성 4.2% (위험대비 0.54) (달 간격) · 최대낙폭 -3% · 보수 0.36% · 가장 나쁜 창 연2.6%</t>
         </is>
       </c>
     </row>
@@ -11630,22 +11532,22 @@
       </c>
       <c r="C154" s="33" t="inlineStr">
         <is>
-          <t>베어링월지급글로벌하이일드증권자투자신탁[H](채권-재간접형)</t>
+          <t>우리프랭클린미국바이오헬스케어증권자투자신탁(주식-재간접형)</t>
         </is>
       </c>
       <c r="D154" s="33" t="inlineStr">
         <is>
-          <t>해외채권형</t>
+          <t>해외주식형</t>
         </is>
       </c>
       <c r="E154" s="33" t="inlineStr">
         <is>
-          <t>베어링자산운용</t>
+          <t>우리자산운용</t>
         </is>
       </c>
       <c r="F154" s="34" t="inlineStr">
         <is>
-          <t>496억원</t>
+          <t>225억원</t>
         </is>
       </c>
       <c r="G154" s="35" t="inlineStr">
@@ -11655,28 +11557,26 @@
       </c>
       <c r="H154" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I154" s="36" t="n">
-        <v>0.0282</v>
+        <v>0.2481</v>
       </c>
       <c r="J154" s="36" t="n">
-        <v>0.0195</v>
-      </c>
-      <c r="K154" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1977</v>
+      </c>
+      <c r="K154" s="37" t="n">
+        <v>-0.1625</v>
       </c>
       <c r="L154" s="34" t="inlineStr">
         <is>
-          <t>0.49~1.19%</t>
+          <t>0.14~1.14%</t>
         </is>
       </c>
       <c r="M154" s="38" t="inlineStr">
         <is>
-          <t>5해 연2.8% · 변동성 1.9% (위험대비 0.01) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.49% · 가장 나쁜 창 연2.8%</t>
+          <t>3해 연24.8% · 변동성 19.8% (위험대비 1.11) (달 간격) · 최대낙폭 -16% · 보수 0.14% · 가장 나쁜 창 연24.8%</t>
         </is>
       </c>
     </row>
@@ -11693,22 +11593,22 @@
       </c>
       <c r="C155" s="14" t="inlineStr">
         <is>
-          <t>AB글로벌고수익증권투자신탁(채권-재간접형)</t>
+          <t>KB글로벌코어리츠부동산자투자신탁(재간접형)(H)(운용)</t>
         </is>
       </c>
       <c r="D155" s="14" t="inlineStr">
         <is>
-          <t>해외채권형</t>
+          <t>해외대체</t>
         </is>
       </c>
       <c r="E155" s="14" t="inlineStr">
         <is>
-          <t>얼라이언스번스틴자산운용</t>
+          <t>케이비자산운용</t>
         </is>
       </c>
       <c r="F155" s="28" t="inlineStr">
         <is>
-          <t>1,629억원</t>
+          <t>217억원</t>
         </is>
       </c>
       <c r="G155" s="30" t="inlineStr">
@@ -11718,28 +11618,26 @@
       </c>
       <c r="H155" s="30" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I155" s="29" t="n">
-        <v>0.0177</v>
+        <v>0.0573</v>
       </c>
       <c r="J155" s="29" t="n">
-        <v>0.0255</v>
-      </c>
-      <c r="K155" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.1328</v>
+      </c>
+      <c r="K155" s="31" t="n">
+        <v>-0.09609999999999999</v>
       </c>
       <c r="L155" s="28" t="inlineStr">
         <is>
-          <t>0.17~1.17%</t>
+          <t>0.57~1.43%</t>
         </is>
       </c>
       <c r="M155" s="32" t="inlineStr">
         <is>
-          <t>5해 연1.8% · 변동성 2.5% (위험대비 -0.41) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.17% · 가장 나쁜 창 연1.8%</t>
+          <t>3해 연5.7% · 변동성 13.3% (위험대비 0.22) (달 간격) · 최대낙폭 -10% · 보수 0.57% · 가장 나쁜 창 연5.7%</t>
         </is>
       </c>
     </row>
@@ -11756,22 +11654,22 @@
       </c>
       <c r="C156" s="33" t="inlineStr">
         <is>
-          <t>한국밸류글로벌배당인컴증권자투자신탁(주식)(모)</t>
+          <t>iM에셋글로벌자산배분증권투자신탁(주식혼합-재간접형)(H)</t>
         </is>
       </c>
       <c r="D156" s="33" t="inlineStr">
         <is>
-          <t>해외주식형</t>
+          <t>해외혼합형</t>
         </is>
       </c>
       <c r="E156" s="33" t="inlineStr">
         <is>
-          <t>한국투자밸류자산운용</t>
+          <t>아이엠에셋자산운용</t>
         </is>
       </c>
       <c r="F156" s="34" t="inlineStr">
         <is>
-          <t>210억원</t>
+          <t>176억원</t>
         </is>
       </c>
       <c r="G156" s="35" t="inlineStr">
@@ -11781,28 +11679,26 @@
       </c>
       <c r="H156" s="35" t="inlineStr">
         <is>
-          <t>5해</t>
+          <t>3해</t>
         </is>
       </c>
       <c r="I156" s="36" t="n">
-        <v>0.1225</v>
+        <v>0.1046</v>
       </c>
       <c r="J156" s="36" t="n">
-        <v>0.1009</v>
-      </c>
-      <c r="K156" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.09660000000000001</v>
+      </c>
+      <c r="K156" s="37" t="n">
+        <v>-0.0765</v>
       </c>
       <c r="L156" s="34" t="inlineStr">
         <is>
-          <t>0.91~1.88%</t>
+          <t>0.80~2.07%</t>
         </is>
       </c>
       <c r="M156" s="38" t="inlineStr">
         <is>
-          <t>5해 연12.2% · 변동성 10.1% (위험대비 0.94) (원천 제공) · 최대낙폭은 못 쟀습니다 · 보수 0.91% · 가장 나쁜 창 연6.2%</t>
+          <t>3해 연10.5% · 변동성 9.7% (위험대비 0.79) (달 간격) · 최대낙폭 -8% · 보수 0.80% · 가장 나쁜 창 연10.5%</t>
         </is>
       </c>
     </row>
@@ -11946,7 +11842,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E7" s="41" t="inlineStr"/>
@@ -12402,11 +12298,11 @@
         </is>
       </c>
       <c r="B30" s="39" t="n">
-        <v>0.0553</v>
+        <v>0.0535</v>
       </c>
       <c r="C30" s="45" t="inlineStr">
         <is>
-          <t>국내채권 40% · 국내주식 40% · 대체 20%</t>
+          <t>대체 40% · 국내채권 30% · 국내주식 30%</t>
         </is>
       </c>
       <c r="D30" s="46" t="n"/>
@@ -12423,7 +12319,7 @@
       </c>
       <c r="C31" s="45" t="inlineStr">
         <is>
-          <t>해외주식 40% · 해외채권 40% · 대체 20%</t>
+          <t>해외채권 40% · 해외주식 40% · 대체 20%</t>
         </is>
       </c>
       <c r="D31" s="46" t="n"/>

</xml_diff>